<commit_message>
Remove emoji characters from marketing calendar and regenerate Excel
https://claude.ai/code/session_01FNPFF5mFSuHNsmFNUSkkTX
</commit_message>
<xml_diff>
--- a/2026_글로벌마케팅캘린더.xlsx
+++ b/2026_글로벌마케팅캘린더.xlsx
@@ -1097,7 +1097,7 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>★ 월별 주요 이벤트</t>
+          <t xml:space="preserve"> 월별 주요 이벤트</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>618🔥</t>
+          <t>618</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>중추절🔥</t>
+          <t>중추절</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>광군절·블프🔥🔥</t>
+          <t>광군절·블프</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -1261,7 +1261,7 @@
       <c r="A5" s="10" t="inlineStr"/>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>🌐 글로벌 인스타그램 공식계정 운영</t>
+          <t xml:space="preserve"> 글로벌 인스타그램 공식계정 운영</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>▶ 목표: 1차목표: 오프라인 판매량 증대 + CGF 브랜드 전문성 구축 | ★ 대표 3개월 1회 현지 직접 방문</t>
+          <t>▶ 목표: 1차목표: 오프라인 판매량 증대 + CGF 브랜드 전문성 구축 |  대표 3개월 1회 현지 직접 방문</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       <c r="A8" s="22" t="inlineStr"/>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>📱 [하이하이] P-Max 연계 디지털 광고</t>
+          <t xml:space="preserve"> [하이하이] P-Max 연계 디지털 광고</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
@@ -1417,7 +1417,7 @@
       <c r="A9" s="22" t="inlineStr"/>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>🔬 CGF 전문성 (의사협회 논문 + KOL/KOC)</t>
+          <t xml:space="preserve"> CGF 전문성 (의사협회 논문 + KOL/KOC)</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
@@ -1455,7 +1455,7 @@
       <c r="A10" s="22" t="inlineStr"/>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>🏪 오프라인 엔드매대 + 시음행사</t>
+          <t xml:space="preserve"> 오프라인 엔드매대 + 시음행사</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -1497,7 +1497,7 @@
       <c r="A11" s="22" t="inlineStr"/>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>🏥 이너샵 VMD + 홍보물 + 온라인</t>
+          <t xml:space="preserve"> 이너샵 VMD + 홍보물 + 온라인</t>
         </is>
       </c>
       <c r="C11" s="24" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>▶ 목표: 최종목표: 코스트코 데모 행사 효율 향상 + 뉴케어 지속 운영 | ★ 6/5 활동 시작</t>
+          <t>▶ 목표: 최종목표: 코스트코 데모 행사 효율 향상 + 뉴케어 지속 운영 |  6/5 활동 시작</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       <c r="A14" s="31" t="inlineStr"/>
       <c r="B14" s="32" t="inlineStr">
         <is>
-          <t>📸 인플루언서 마케팅 (인스타+광고코드+현장스케치 영상)</t>
+          <t xml:space="preserve"> 인플루언서 마케팅 (인스타+광고코드+현장스케치 영상)</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
@@ -1625,7 +1625,7 @@
       <c r="A15" s="31" t="inlineStr"/>
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>📲 뉴케어 일본 인스타 브랜드페이지 + 체험단</t>
+          <t xml:space="preserve"> 뉴케어 일본 인스타 브랜드페이지 + 체험단</t>
         </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
@@ -1667,7 +1667,7 @@
       <c r="A16" s="31" t="inlineStr"/>
       <c r="B16" s="32" t="inlineStr">
         <is>
-          <t>🥣 칼비 후루그라 코스트코 공동 샘플링 협업</t>
+          <t xml:space="preserve"> 칼비 후루그라 코스트코 공동 샘플링 협업</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
@@ -1699,7 +1699,7 @@
       <c r="A17" s="31" t="inlineStr"/>
       <c r="B17" s="32" t="inlineStr">
         <is>
-          <t>🛒 홈쇼핑/라이브커머스/온라인 오픈 SA·DA</t>
+          <t xml:space="preserve"> 홈쇼핑/라이브커머스/온라인 오픈 SA·DA</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
@@ -1785,7 +1785,7 @@
       <c r="A20" s="39" t="inlineStr"/>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>🏬 브랜드 전용존 구축 + 현장 시음 진행</t>
+          <t xml:space="preserve"> 브랜드 전용존 구축 + 현장 시음 진행</t>
         </is>
       </c>
       <c r="C20" s="41" t="inlineStr">
@@ -1819,7 +1819,7 @@
       <c r="A21" s="39" t="inlineStr"/>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>🛍️ 블랙프라이데이·Cyber Monday 이벤트</t>
+          <t>️ 블랙프라이데이·Cyber Monday 이벤트</t>
         </is>
       </c>
       <c r="C21" s="41" t="inlineStr">
@@ -1853,7 +1853,7 @@
       <c r="A22" s="39" t="inlineStr"/>
       <c r="B22" s="40" t="inlineStr">
         <is>
-          <t>📦 헤이N 브랜드 아마존 테스트 광고</t>
+          <t xml:space="preserve"> 헤이N 브랜드 아마존 테스트 광고</t>
         </is>
       </c>
       <c r="C22" s="41" t="inlineStr">
@@ -1947,7 +1947,7 @@
       <c r="A25" s="47" t="inlineStr"/>
       <c r="B25" s="48" t="inlineStr">
         <is>
-          <t>🛒 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
+          <t xml:space="preserve"> 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
         </is>
       </c>
       <c r="C25" s="49" t="inlineStr">
@@ -1977,7 +1977,7 @@
       <c r="A26" s="47" t="inlineStr"/>
       <c r="B26" s="48" t="inlineStr">
         <is>
-          <t>🎬 KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
+          <t xml:space="preserve"> KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
         </is>
       </c>
       <c r="C26" s="49" t="inlineStr">
@@ -2013,7 +2013,7 @@
       <c r="A27" s="47" t="inlineStr"/>
       <c r="B27" s="48" t="inlineStr">
         <is>
-          <t>🎉 광군절 11.11 집중 캠페인</t>
+          <t xml:space="preserve"> 광군절 11.11 집중 캠페인</t>
         </is>
       </c>
       <c r="C27" s="49" t="inlineStr">
@@ -2045,7 +2045,7 @@
       <c r="A28" s="47" t="inlineStr"/>
       <c r="B28" s="48" t="inlineStr">
         <is>
-          <t>🛒 쌍12 (12/12) 연말 마감 캠페인</t>
+          <t xml:space="preserve"> 쌍12 (12/12) 연말 마감 캠페인</t>
         </is>
       </c>
       <c r="C28" s="49" t="inlineStr">
@@ -2129,7 +2129,7 @@
       <c r="A31" s="53" t="inlineStr"/>
       <c r="B31" s="54" t="inlineStr">
         <is>
-          <t>☀️ 여름 음료 성수기 집중 광고 (7~9월)</t>
+          <t>️ 여름 음료 성수기 집중 광고 (7~9월)</t>
         </is>
       </c>
       <c r="C31" s="55" t="inlineStr">
@@ -2163,7 +2163,7 @@
       <c r="A32" s="53" t="inlineStr"/>
       <c r="B32" s="54" t="inlineStr">
         <is>
-          <t>💊 Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
+          <t xml:space="preserve"> Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
         </is>
       </c>
       <c r="C32" s="55" t="inlineStr">
@@ -2245,7 +2245,7 @@
       <c r="A35" s="60" t="inlineStr"/>
       <c r="B35" s="61" t="inlineStr">
         <is>
-          <t>🏃 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
+          <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
         </is>
       </c>
       <c r="C35" s="62" t="inlineStr">
@@ -2325,7 +2325,7 @@
       <c r="A38" s="66" t="inlineStr"/>
       <c r="B38" s="67" t="inlineStr">
         <is>
-          <t>🤝 가디언 협업 확대 + 미팅 후 입점 지원</t>
+          <t xml:space="preserve"> 가디언 협업 확대 + 미팅 후 입점 지원</t>
         </is>
       </c>
       <c r="C38" s="68" t="inlineStr">
@@ -2357,7 +2357,7 @@
       <c r="A39" s="66" t="inlineStr"/>
       <c r="B39" s="67" t="inlineStr">
         <is>
-          <t>🏢 현지 박람회 / 전시회 참가</t>
+          <t xml:space="preserve"> 현지 박람회 / 전시회 참가</t>
         </is>
       </c>
       <c r="C39" s="68" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="B41" s="72" t="inlineStr">
         <is>
-          <t>▶ 목표: ★ 시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
+          <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2433,7 @@
       <c r="A42" s="73" t="inlineStr"/>
       <c r="B42" s="74" t="inlineStr">
         <is>
-          <t>📉 Dermazone 최소 프로모 지원</t>
+          <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
         </is>
       </c>
       <c r="C42" s="75" t="inlineStr">
@@ -2513,7 +2513,7 @@
       <c r="A45" s="81" t="inlineStr"/>
       <c r="B45" s="82" t="inlineStr">
         <is>
-          <t>🦘 천호케어 + 대상 호주 공동 마케팅 지원</t>
+          <t xml:space="preserve"> 천호케어 + 대상 호주 공동 마케팅 지원</t>
         </is>
       </c>
       <c r="C45" s="83" t="inlineStr">

</xml_diff>

<commit_message>
Update marketing calendar: Vietnam P-Max 3억 (Aug/Oct focus), China 화룬강중 launch, Mongolia insert video
- Vietnam P-Max redistributed to 300M total: Aug relaunch focus (100M), Oct Newcare focus (80M)
- China: added 화룬강중 (new) 40M launch support for 800M pipeline
- Mongolia: added 50M insert video production replacing Vietnam Golden channel
- Total budget maintained at 1,500M KRW

https://claude.ai/code/session_01FNPFF5mFSuHNsmFNUSkkTX
</commit_message>
<xml_diff>
--- a/2026_글로벌마케팅캘린더.xlsx
+++ b/2026_글로벌마케팅캘린더.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>구글 P-Max+쇼피 연동 / 키성장 타겟</t>
+          <t>8월 리뉴얼 런칭 집중 / 10월 뉴케어 집중 / 총 3억</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr"/>
@@ -1391,26 +1391,26 @@
       <c r="G8" s="25" t="inlineStr"/>
       <c r="H8" s="25" t="inlineStr"/>
       <c r="I8" s="26" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="J8" s="26" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="K8" s="26" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="L8" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="M8" s="26" t="n">
         <v>80</v>
       </c>
-      <c r="M8" s="26" t="n">
+      <c r="N8" s="26" t="n">
         <v>30</v>
-      </c>
-      <c r="N8" s="26" t="n">
-        <v>20</v>
       </c>
       <c r="O8" s="25" t="inlineStr"/>
       <c r="P8" s="27" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -1543,28 +1543,28 @@
       <c r="G12" s="18" t="inlineStr"/>
       <c r="H12" s="18" t="inlineStr"/>
       <c r="I12" s="18" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="K12" s="18" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="L12" s="18" t="n">
-        <v>115</v>
+        <v>55</v>
       </c>
       <c r="M12" s="18" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="N12" s="18" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O12" s="18" t="n">
         <v>10</v>
       </c>
       <c r="P12" s="19" t="n">
-        <v>570</v>
+        <v>480</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B24" s="46" t="inlineStr">
         <is>
-          <t>▶ 목표: 최종목표: 역직구 채널 안정화 + FSMP Top5 진입</t>
+          <t>▶ 목표: 최종목표: 역직구 채널 안정화 + GP Top5 진입 | 화룬강중 신규 800 파이프라인 런칭</t>
         </is>
       </c>
     </row>
@@ -2072,103 +2072,103 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="52" t="inlineStr">
+      <c r="A29" s="47" t="inlineStr"/>
+      <c r="B29" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 화룬강중 (신규) 런칭 지원</t>
+        </is>
+      </c>
+      <c r="C29" s="49" t="inlineStr">
+        <is>
+          <t>800 파이프라인 / 런칭 예산 우선 배정 / 케이코스메몰 축소분 재배분</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr"/>
+      <c r="E29" s="25" t="inlineStr"/>
+      <c r="F29" s="25" t="inlineStr"/>
+      <c r="G29" s="25" t="inlineStr"/>
+      <c r="H29" s="25" t="inlineStr"/>
+      <c r="I29" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="J29" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="K29" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L29" s="25" t="inlineStr"/>
+      <c r="M29" s="25" t="inlineStr"/>
+      <c r="N29" s="25" t="inlineStr"/>
+      <c r="O29" s="25" t="inlineStr"/>
+      <c r="P29" s="51" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="52" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C29" s="17" t="inlineStr"/>
-      <c r="D29" s="18" t="inlineStr"/>
-      <c r="E29" s="18" t="inlineStr"/>
-      <c r="F29" s="18" t="inlineStr"/>
-      <c r="G29" s="18" t="inlineStr"/>
-      <c r="H29" s="18" t="inlineStr"/>
-      <c r="I29" s="18" t="n">
+      <c r="C30" s="17" t="inlineStr"/>
+      <c r="D30" s="18" t="inlineStr"/>
+      <c r="E30" s="18" t="inlineStr"/>
+      <c r="F30" s="18" t="inlineStr"/>
+      <c r="G30" s="18" t="inlineStr"/>
+      <c r="H30" s="18" t="inlineStr"/>
+      <c r="I30" s="18" t="n">
+        <v>80</v>
+      </c>
+      <c r="J30" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="K30" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="L30" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="M30" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="N30" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="J29" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="K29" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="L29" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="M29" s="18" t="n">
+      <c r="O30" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="N29" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="O29" s="18" t="n">
-        <v>30</v>
-      </c>
-      <c r="P29" s="19" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="P30" s="19" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>대만</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 음료시장 성수기 집중 + Medfirst FSMP Top3 달성</t>
         </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="53" t="inlineStr"/>
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t>️ 여름 음료 성수기 집중 광고 (7~9월)</t>
-        </is>
-      </c>
-      <c r="C31" s="55" t="inlineStr">
-        <is>
-          <t>여름 건강음료 수요 피크 시즌</t>
-        </is>
-      </c>
-      <c r="D31" s="25" t="inlineStr"/>
-      <c r="E31" s="25" t="inlineStr"/>
-      <c r="F31" s="25" t="inlineStr"/>
-      <c r="G31" s="25" t="inlineStr"/>
-      <c r="H31" s="25" t="inlineStr"/>
-      <c r="I31" s="25" t="inlineStr"/>
-      <c r="J31" s="56" t="n">
-        <v>20</v>
-      </c>
-      <c r="K31" s="56" t="n">
-        <v>25</v>
-      </c>
-      <c r="L31" s="56" t="n">
-        <v>15</v>
-      </c>
-      <c r="M31" s="25" t="inlineStr"/>
-      <c r="N31" s="25" t="inlineStr"/>
-      <c r="O31" s="25" t="inlineStr"/>
-      <c r="P31" s="57" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="53" t="inlineStr"/>
       <c r="B32" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
+          <t>️ 여름 음료 성수기 집중 광고 (7~9월)</t>
         </is>
       </c>
       <c r="C32" s="55" t="inlineStr">
         <is>
-          <t>닥터 추천 마크 부착 후 집행</t>
+          <t>여름 건강음료 수요 피크 시즌</t>
         </is>
       </c>
       <c r="D32" s="25" t="inlineStr"/>
@@ -2177,474 +2177,546 @@
       <c r="G32" s="25" t="inlineStr"/>
       <c r="H32" s="25" t="inlineStr"/>
       <c r="I32" s="25" t="inlineStr"/>
-      <c r="J32" s="25" t="inlineStr"/>
-      <c r="K32" s="25" t="inlineStr"/>
-      <c r="L32" s="25" t="inlineStr"/>
-      <c r="M32" s="56" t="n">
-        <v>10</v>
-      </c>
+      <c r="J32" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="K32" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="L32" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="M32" s="25" t="inlineStr"/>
       <c r="N32" s="25" t="inlineStr"/>
-      <c r="O32" s="56" t="n">
-        <v>10</v>
-      </c>
+      <c r="O32" s="25" t="inlineStr"/>
       <c r="P32" s="57" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="53" t="inlineStr"/>
+      <c r="B33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
+        </is>
+      </c>
+      <c r="C33" s="55" t="inlineStr">
+        <is>
+          <t>닥터 추천 마크 부착 후 집행</t>
+        </is>
+      </c>
+      <c r="D33" s="25" t="inlineStr"/>
+      <c r="E33" s="25" t="inlineStr"/>
+      <c r="F33" s="25" t="inlineStr"/>
+      <c r="G33" s="25" t="inlineStr"/>
+      <c r="H33" s="25" t="inlineStr"/>
+      <c r="I33" s="25" t="inlineStr"/>
+      <c r="J33" s="25" t="inlineStr"/>
+      <c r="K33" s="25" t="inlineStr"/>
+      <c r="L33" s="25" t="inlineStr"/>
+      <c r="M33" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="N33" s="25" t="inlineStr"/>
+      <c r="O33" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="P33" s="57" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="28" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="28" t="inlineStr">
         <is>
           <t>대만</t>
         </is>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C33" s="17" t="inlineStr"/>
-      <c r="D33" s="18" t="inlineStr"/>
-      <c r="E33" s="18" t="inlineStr"/>
-      <c r="F33" s="18" t="inlineStr"/>
-      <c r="G33" s="18" t="inlineStr"/>
-      <c r="H33" s="18" t="inlineStr"/>
-      <c r="I33" s="18" t="inlineStr"/>
-      <c r="J33" s="18" t="n">
+      <c r="C34" s="17" t="inlineStr"/>
+      <c r="D34" s="18" t="inlineStr"/>
+      <c r="E34" s="18" t="inlineStr"/>
+      <c r="F34" s="18" t="inlineStr"/>
+      <c r="G34" s="18" t="inlineStr"/>
+      <c r="H34" s="18" t="inlineStr"/>
+      <c r="I34" s="18" t="inlineStr"/>
+      <c r="J34" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K33" s="18" t="n">
+      <c r="K34" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="L33" s="18" t="n">
+      <c r="L34" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="M33" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="N33" s="18" t="inlineStr"/>
-      <c r="O33" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P33" s="19" t="n">
+      <c r="M34" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="N34" s="18" t="inlineStr"/>
+      <c r="O34" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P34" s="19" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="58" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="58" t="inlineStr">
         <is>
           <t>몽골</t>
         </is>
       </c>
-      <c r="B34" s="59" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 현지 자체 브랜딩 지원 + 스포츠 마케팅 강화</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="60" t="inlineStr"/>
-      <c r="B35" s="61" t="inlineStr">
+      <c r="B35" s="59" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 현지 자체 브랜딩 지원 + 스포츠 마케팅 강화 | 베트남 골든 없음 → 인서트 영상 지원 전환</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="60" t="inlineStr"/>
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
         </is>
       </c>
-      <c r="C35" s="62" t="inlineStr">
+      <c r="C36" s="62" t="inlineStr">
         <is>
           <t>현지 파트너 주도 / 웰라이프 지원</t>
         </is>
       </c>
-      <c r="D35" s="25" t="inlineStr"/>
-      <c r="E35" s="25" t="inlineStr"/>
-      <c r="F35" s="25" t="inlineStr"/>
-      <c r="G35" s="25" t="inlineStr"/>
-      <c r="H35" s="25" t="inlineStr"/>
-      <c r="I35" s="63" t="n">
+      <c r="D36" s="25" t="inlineStr"/>
+      <c r="E36" s="25" t="inlineStr"/>
+      <c r="F36" s="25" t="inlineStr"/>
+      <c r="G36" s="25" t="inlineStr"/>
+      <c r="H36" s="25" t="inlineStr"/>
+      <c r="I36" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="J35" s="25" t="inlineStr"/>
-      <c r="K35" s="25" t="inlineStr"/>
-      <c r="L35" s="63" t="n">
+      <c r="J36" s="25" t="inlineStr"/>
+      <c r="K36" s="25" t="inlineStr"/>
+      <c r="L36" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="M35" s="25" t="inlineStr"/>
-      <c r="N35" s="25" t="inlineStr"/>
-      <c r="O35" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="P35" s="64" t="n">
+      <c r="M36" s="25" t="inlineStr"/>
+      <c r="N36" s="25" t="inlineStr"/>
+      <c r="O36" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="P36" s="64" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="65" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="60" t="inlineStr"/>
+      <c r="B37" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 인서트 영상 제작 + 현지 배포 지원</t>
+        </is>
+      </c>
+      <c r="C37" s="62" t="inlineStr">
+        <is>
+          <t>베트남 골든 채널 종료 → 몽골 자체 SNS 인서트로 전환</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr"/>
+      <c r="E37" s="25" t="inlineStr"/>
+      <c r="F37" s="25" t="inlineStr"/>
+      <c r="G37" s="25" t="inlineStr"/>
+      <c r="H37" s="25" t="inlineStr"/>
+      <c r="I37" s="25" t="inlineStr"/>
+      <c r="J37" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="K37" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="L37" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="M37" s="25" t="inlineStr"/>
+      <c r="N37" s="25" t="inlineStr"/>
+      <c r="O37" s="25" t="inlineStr"/>
+      <c r="P37" s="64" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="65" t="inlineStr">
         <is>
           <t>몽골</t>
         </is>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr"/>
-      <c r="D36" s="18" t="inlineStr"/>
-      <c r="E36" s="18" t="inlineStr"/>
-      <c r="F36" s="18" t="inlineStr"/>
-      <c r="G36" s="18" t="inlineStr"/>
-      <c r="H36" s="18" t="inlineStr"/>
-      <c r="I36" s="18" t="n">
+      <c r="C38" s="17" t="inlineStr"/>
+      <c r="D38" s="18" t="inlineStr"/>
+      <c r="E38" s="18" t="inlineStr"/>
+      <c r="F38" s="18" t="inlineStr"/>
+      <c r="G38" s="18" t="inlineStr"/>
+      <c r="H38" s="18" t="inlineStr"/>
+      <c r="I38" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J36" s="18" t="inlineStr"/>
-      <c r="K36" s="18" t="inlineStr"/>
-      <c r="L36" s="18" t="n">
+      <c r="J38" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="K38" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="L38" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="M38" s="18" t="inlineStr"/>
+      <c r="N38" s="18" t="inlineStr"/>
+      <c r="O38" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P38" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="58" t="inlineStr">
+        <is>
+          <t>싱가포르</t>
+        </is>
+      </c>
+      <c r="B39" s="59" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 가디언 입점 매출 확대 + 박람회 신규 채널 개척</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="66" t="inlineStr"/>
+      <c r="B40" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 가디언 협업 확대 + 미팅 후 입점 지원</t>
+        </is>
+      </c>
+      <c r="C40" s="68" t="inlineStr">
+        <is>
+          <t>가디언 83개점 → 확장 공략</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="inlineStr"/>
+      <c r="E40" s="25" t="inlineStr"/>
+      <c r="F40" s="25" t="inlineStr"/>
+      <c r="G40" s="25" t="inlineStr"/>
+      <c r="H40" s="25" t="inlineStr"/>
+      <c r="I40" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="J40" s="25" t="inlineStr"/>
+      <c r="K40" s="25" t="inlineStr"/>
+      <c r="L40" s="25" t="inlineStr"/>
+      <c r="M40" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="N40" s="25" t="inlineStr"/>
+      <c r="O40" s="25" t="inlineStr"/>
+      <c r="P40" s="70" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="66" t="inlineStr"/>
+      <c r="B41" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 현지 박람회 / 전시회 참가</t>
+        </is>
+      </c>
+      <c r="C41" s="68" t="inlineStr">
+        <is>
+          <t>신규 바이어 발굴</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="inlineStr"/>
+      <c r="E41" s="25" t="inlineStr"/>
+      <c r="F41" s="25" t="inlineStr"/>
+      <c r="G41" s="25" t="inlineStr"/>
+      <c r="H41" s="25" t="inlineStr"/>
+      <c r="I41" s="25" t="inlineStr"/>
+      <c r="J41" s="25" t="inlineStr"/>
+      <c r="K41" s="25" t="inlineStr"/>
+      <c r="L41" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="M41" s="25" t="inlineStr"/>
+      <c r="N41" s="25" t="inlineStr"/>
+      <c r="O41" s="25" t="inlineStr"/>
+      <c r="P41" s="70" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="65" t="inlineStr">
+        <is>
+          <t>싱가포르</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>소계</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr"/>
+      <c r="D42" s="18" t="inlineStr"/>
+      <c r="E42" s="18" t="inlineStr"/>
+      <c r="F42" s="18" t="inlineStr"/>
+      <c r="G42" s="18" t="inlineStr"/>
+      <c r="H42" s="18" t="inlineStr"/>
+      <c r="I42" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="J42" s="18" t="inlineStr"/>
+      <c r="K42" s="18" t="inlineStr"/>
+      <c r="L42" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="M42" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="N42" s="18" t="inlineStr"/>
+      <c r="O42" s="18" t="inlineStr"/>
+      <c r="P42" s="19" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="71" t="inlineStr">
+        <is>
+          <t>중동</t>
+        </is>
+      </c>
+      <c r="B43" s="72" t="inlineStr">
+        <is>
+          <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="73" t="inlineStr"/>
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
+        </is>
+      </c>
+      <c r="C44" s="75" t="inlineStr">
+        <is>
+          <t>현상 유지 / 추가 투자 없음</t>
+        </is>
+      </c>
+      <c r="D44" s="25" t="inlineStr"/>
+      <c r="E44" s="25" t="inlineStr"/>
+      <c r="F44" s="25" t="inlineStr"/>
+      <c r="G44" s="25" t="inlineStr"/>
+      <c r="H44" s="25" t="inlineStr"/>
+      <c r="I44" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="M36" s="18" t="inlineStr"/>
-      <c r="N36" s="18" t="inlineStr"/>
-      <c r="O36" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P36" s="19" t="n">
+      <c r="J44" s="25" t="inlineStr"/>
+      <c r="K44" s="25" t="inlineStr"/>
+      <c r="L44" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="M44" s="25" t="inlineStr"/>
+      <c r="N44" s="25" t="inlineStr"/>
+      <c r="O44" s="76" t="n">
+        <v>10</v>
+      </c>
+      <c r="P44" s="77" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="58" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="B37" s="59" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 가디언 입점 매출 확대 + 박람회 신규 채널 개척</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="66" t="inlineStr"/>
-      <c r="B38" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 가디언 협업 확대 + 미팅 후 입점 지원</t>
-        </is>
-      </c>
-      <c r="C38" s="68" t="inlineStr">
-        <is>
-          <t>가디언 83개점 → 확장 공략</t>
-        </is>
-      </c>
-      <c r="D38" s="25" t="inlineStr"/>
-      <c r="E38" s="25" t="inlineStr"/>
-      <c r="F38" s="25" t="inlineStr"/>
-      <c r="G38" s="25" t="inlineStr"/>
-      <c r="H38" s="25" t="inlineStr"/>
-      <c r="I38" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="J38" s="25" t="inlineStr"/>
-      <c r="K38" s="25" t="inlineStr"/>
-      <c r="L38" s="25" t="inlineStr"/>
-      <c r="M38" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="N38" s="25" t="inlineStr"/>
-      <c r="O38" s="25" t="inlineStr"/>
-      <c r="P38" s="70" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="66" t="inlineStr"/>
-      <c r="B39" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 현지 박람회 / 전시회 참가</t>
-        </is>
-      </c>
-      <c r="C39" s="68" t="inlineStr">
-        <is>
-          <t>신규 바이어 발굴</t>
-        </is>
-      </c>
-      <c r="D39" s="25" t="inlineStr"/>
-      <c r="E39" s="25" t="inlineStr"/>
-      <c r="F39" s="25" t="inlineStr"/>
-      <c r="G39" s="25" t="inlineStr"/>
-      <c r="H39" s="25" t="inlineStr"/>
-      <c r="I39" s="25" t="inlineStr"/>
-      <c r="J39" s="25" t="inlineStr"/>
-      <c r="K39" s="25" t="inlineStr"/>
-      <c r="L39" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="M39" s="25" t="inlineStr"/>
-      <c r="N39" s="25" t="inlineStr"/>
-      <c r="O39" s="25" t="inlineStr"/>
-      <c r="P39" s="70" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="65" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="B40" s="16" t="inlineStr">
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="78" t="inlineStr">
+        <is>
+          <t>중동</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr"/>
-      <c r="D40" s="18" t="inlineStr"/>
-      <c r="E40" s="18" t="inlineStr"/>
-      <c r="F40" s="18" t="inlineStr"/>
-      <c r="G40" s="18" t="inlineStr"/>
-      <c r="H40" s="18" t="inlineStr"/>
-      <c r="I40" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="J40" s="18" t="inlineStr"/>
-      <c r="K40" s="18" t="inlineStr"/>
-      <c r="L40" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="M40" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="N40" s="18" t="inlineStr"/>
-      <c r="O40" s="18" t="inlineStr"/>
-      <c r="P40" s="19" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="71" t="inlineStr">
-        <is>
-          <t>중동</t>
-        </is>
-      </c>
-      <c r="B41" s="72" t="inlineStr">
-        <is>
-          <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="73" t="inlineStr"/>
-      <c r="B42" s="74" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
-        </is>
-      </c>
-      <c r="C42" s="75" t="inlineStr">
-        <is>
-          <t>현상 유지 / 추가 투자 없음</t>
-        </is>
-      </c>
-      <c r="D42" s="25" t="inlineStr"/>
-      <c r="E42" s="25" t="inlineStr"/>
-      <c r="F42" s="25" t="inlineStr"/>
-      <c r="G42" s="25" t="inlineStr"/>
-      <c r="H42" s="25" t="inlineStr"/>
-      <c r="I42" s="76" t="n">
+      <c r="C45" s="17" t="inlineStr"/>
+      <c r="D45" s="18" t="inlineStr"/>
+      <c r="E45" s="18" t="inlineStr"/>
+      <c r="F45" s="18" t="inlineStr"/>
+      <c r="G45" s="18" t="inlineStr"/>
+      <c r="H45" s="18" t="inlineStr"/>
+      <c r="I45" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J42" s="25" t="inlineStr"/>
-      <c r="K42" s="25" t="inlineStr"/>
-      <c r="L42" s="76" t="n">
+      <c r="J45" s="18" t="inlineStr"/>
+      <c r="K45" s="18" t="inlineStr"/>
+      <c r="L45" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M42" s="25" t="inlineStr"/>
-      <c r="N42" s="25" t="inlineStr"/>
-      <c r="O42" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="P42" s="77" t="n">
+      <c r="M45" s="18" t="inlineStr"/>
+      <c r="N45" s="18" t="inlineStr"/>
+      <c r="O45" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P45" s="19" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="78" t="inlineStr">
-        <is>
-          <t>중동</t>
-        </is>
-      </c>
-      <c r="B43" s="16" t="inlineStr">
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="79" t="inlineStr">
+        <is>
+          <t>호주</t>
+        </is>
+      </c>
+      <c r="B46" s="80" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 천호케어 파트너십 유지 + 대상 호주 채널 안정화</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="81" t="inlineStr"/>
+      <c r="B47" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 천호케어 + 대상 호주 공동 마케팅 지원</t>
+        </is>
+      </c>
+      <c r="C47" s="83" t="inlineStr">
+        <is>
+          <t>파트너 요청 시 지원</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="inlineStr"/>
+      <c r="E47" s="25" t="inlineStr"/>
+      <c r="F47" s="25" t="inlineStr"/>
+      <c r="G47" s="25" t="inlineStr"/>
+      <c r="H47" s="25" t="inlineStr"/>
+      <c r="I47" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" s="25" t="inlineStr"/>
+      <c r="K47" s="25" t="inlineStr"/>
+      <c r="L47" s="84" t="n">
+        <v>10</v>
+      </c>
+      <c r="M47" s="25" t="inlineStr"/>
+      <c r="N47" s="25" t="inlineStr"/>
+      <c r="O47" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="P47" s="85" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="86" t="inlineStr">
+        <is>
+          <t>호주</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr"/>
-      <c r="D43" s="18" t="inlineStr"/>
-      <c r="E43" s="18" t="inlineStr"/>
-      <c r="F43" s="18" t="inlineStr"/>
-      <c r="G43" s="18" t="inlineStr"/>
-      <c r="H43" s="18" t="inlineStr"/>
-      <c r="I43" s="18" t="n">
+      <c r="C48" s="17" t="inlineStr"/>
+      <c r="D48" s="18" t="inlineStr"/>
+      <c r="E48" s="18" t="inlineStr"/>
+      <c r="F48" s="18" t="inlineStr"/>
+      <c r="G48" s="18" t="inlineStr"/>
+      <c r="H48" s="18" t="inlineStr"/>
+      <c r="I48" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J43" s="18" t="inlineStr"/>
-      <c r="K43" s="18" t="inlineStr"/>
-      <c r="L43" s="18" t="n">
+      <c r="J48" s="18" t="inlineStr"/>
+      <c r="K48" s="18" t="inlineStr"/>
+      <c r="L48" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="M48" s="18" t="inlineStr"/>
+      <c r="N48" s="18" t="inlineStr"/>
+      <c r="O48" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M43" s="18" t="inlineStr"/>
-      <c r="N43" s="18" t="inlineStr"/>
-      <c r="O43" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P43" s="19" t="n">
+      <c r="P48" s="19" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="79" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="B44" s="80" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 천호케어 파트너십 유지 + 대상 호주 채널 안정화</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="81" t="inlineStr"/>
-      <c r="B45" s="82" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 천호케어 + 대상 호주 공동 마케팅 지원</t>
-        </is>
-      </c>
-      <c r="C45" s="83" t="inlineStr">
-        <is>
-          <t>파트너 요청 시 지원</t>
-        </is>
-      </c>
-      <c r="D45" s="25" t="inlineStr"/>
-      <c r="E45" s="25" t="inlineStr"/>
-      <c r="F45" s="25" t="inlineStr"/>
-      <c r="G45" s="25" t="inlineStr"/>
-      <c r="H45" s="25" t="inlineStr"/>
-      <c r="I45" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="J45" s="25" t="inlineStr"/>
-      <c r="K45" s="25" t="inlineStr"/>
-      <c r="L45" s="84" t="n">
-        <v>10</v>
-      </c>
-      <c r="M45" s="25" t="inlineStr"/>
-      <c r="N45" s="25" t="inlineStr"/>
-      <c r="O45" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="P45" s="85" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="86" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>소계</t>
-        </is>
-      </c>
-      <c r="C46" s="17" t="inlineStr"/>
-      <c r="D46" s="18" t="inlineStr"/>
-      <c r="E46" s="18" t="inlineStr"/>
-      <c r="F46" s="18" t="inlineStr"/>
-      <c r="G46" s="18" t="inlineStr"/>
-      <c r="H46" s="18" t="inlineStr"/>
-      <c r="I46" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J46" s="18" t="inlineStr"/>
-      <c r="K46" s="18" t="inlineStr"/>
-      <c r="L46" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="M46" s="18" t="inlineStr"/>
-      <c r="N46" s="18" t="inlineStr"/>
-      <c r="O46" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="P46" s="19" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="87" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="87" t="inlineStr">
         <is>
           <t>총 합계 (백만원)</t>
         </is>
       </c>
-      <c r="D47" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="E47" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="F47" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="G47" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="H47" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="I47" s="88" t="n">
-        <v>265</v>
-      </c>
-      <c r="J47" s="88" t="n">
-        <v>230</v>
-      </c>
-      <c r="K47" s="88" t="n">
-        <v>270</v>
-      </c>
-      <c r="L47" s="88" t="n">
+      <c r="D49" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="E49" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="F49" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="G49" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="H49" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="I49" s="88" t="n">
         <v>245</v>
       </c>
-      <c r="M47" s="88" t="n">
-        <v>150</v>
-      </c>
-      <c r="N47" s="88" t="n">
-        <v>180</v>
-      </c>
-      <c r="O47" s="88" t="n">
+      <c r="J49" s="88" t="n">
+        <v>220</v>
+      </c>
+      <c r="K49" s="88" t="n">
+        <v>290</v>
+      </c>
+      <c r="L49" s="88" t="n">
+        <v>195</v>
+      </c>
+      <c r="M49" s="88" t="n">
+        <v>200</v>
+      </c>
+      <c r="N49" s="88" t="n">
+        <v>190</v>
+      </c>
+      <c r="O49" s="88" t="n">
         <v>110</v>
       </c>
-      <c r="P47" s="89" t="n">
+      <c r="P49" s="89" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 315  |  하반기(7~12월) 합계: 1,185  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 295  |  하반기(7~12월) 합계: 1,205  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B43:P43"/>
     <mergeCell ref="B7:P7"/>
-    <mergeCell ref="B44:P44"/>
+    <mergeCell ref="B39:P39"/>
     <mergeCell ref="B24:P24"/>
-    <mergeCell ref="B34:P34"/>
-    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="B19:P19"/>
-    <mergeCell ref="B37:P37"/>
-    <mergeCell ref="B41:P41"/>
-    <mergeCell ref="A48:P48"/>
+    <mergeCell ref="B31:P31"/>
+    <mergeCell ref="B46:P46"/>
+    <mergeCell ref="A50:P50"/>
+    <mergeCell ref="B35:P35"/>
     <mergeCell ref="B4:P4"/>
     <mergeCell ref="B13:P13"/>
-    <mergeCell ref="B30:P30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revise Vietnam to 5.95억: P-Max restored, add sampling+LiveCommerce; remove 천호케어
- Vietnam: P-Max contract intact (390M), CGF 50M, add sampling+content 40M, live commerce 35M = 595M
- Japan: reduce 인플루언서 to 90M, 홈쇼핑 to 20M
- Australia: remove 천호케어 (low ROI), direct channel only
- Singapore: focus on EXACTITUDE reorder + Guardian
- 중동: minimize to 5M
- Total maintained at 1,500M KRW

https://claude.ai/code/session_01FNPFF5mFSuHNsmFNUSkkTX
</commit_message>
<xml_diff>
--- a/2026_글로벌마케팅캘린더.xlsx
+++ b/2026_글로벌마케팅캘린더.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P50"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>▶ 목표: 1차목표: 오프라인 판매량 증대 + CGF 브랜드 전문성 구축 |  대표 3개월 1회 현지 직접 방문</t>
+          <t>▶ 목표: 1차목표: 오프라인 판매량 증대 + CGF GP 구축 | 내년 법인화 핵심국가 | 대표 3개월 1회 현지 직접 방문</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>8월 리뉴얼 런칭 집중 / 10월 뉴케어 집중 / 총 3억</t>
+          <t>계약 완료 / 키성장 타겟 / 쇼피 연동</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr"/>
@@ -1391,26 +1391,26 @@
       <c r="G8" s="25" t="inlineStr"/>
       <c r="H8" s="25" t="inlineStr"/>
       <c r="I8" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="J8" s="26" t="n">
+        <v>90</v>
+      </c>
+      <c r="K8" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="L8" s="26" t="n">
+        <v>80</v>
+      </c>
+      <c r="M8" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="N8" s="26" t="n">
         <v>20</v>
-      </c>
-      <c r="J8" s="26" t="n">
-        <v>50</v>
-      </c>
-      <c r="K8" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="L8" s="26" t="n">
-        <v>20</v>
-      </c>
-      <c r="M8" s="26" t="n">
-        <v>80</v>
-      </c>
-      <c r="N8" s="26" t="n">
-        <v>30</v>
       </c>
       <c r="O8" s="25" t="inlineStr"/>
       <c r="P8" s="27" t="n">
-        <v>300</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -1434,21 +1434,21 @@
         <v>20</v>
       </c>
       <c r="J9" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K9" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L9" s="26" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M9" s="26" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N9" s="25" t="inlineStr"/>
       <c r="O9" s="25" t="inlineStr"/>
       <c r="P9" s="27" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>월 1천만 / 윈마트 262개 확장 연동</t>
+          <t>윈마트 262개 확장 / 일본 구조 복사 적용</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr"/>
@@ -1475,10 +1475,10 @@
         <v>10</v>
       </c>
       <c r="K10" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L10" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M10" s="26" t="n">
         <v>10</v>
@@ -1486,11 +1486,9 @@
       <c r="N10" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="O10" s="26" t="n">
-        <v>10</v>
-      </c>
+      <c r="O10" s="25" t="inlineStr"/>
       <c r="P10" s="27" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -1513,7 +1511,7 @@
       <c r="I11" s="25" t="inlineStr"/>
       <c r="J11" s="25" t="inlineStr"/>
       <c r="K11" s="26" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L11" s="26" t="n">
         <v>10</v>
@@ -1522,157 +1520,143 @@
       <c r="N11" s="25" t="inlineStr"/>
       <c r="O11" s="25" t="inlineStr"/>
       <c r="P11" s="27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr"/>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 매장 샘플링 + 온라인 콘텐츠 연계</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>일본 칼비 구조 복사 / 시음→SNS 후기→재구매 루프</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr"/>
+      <c r="E12" s="25" t="inlineStr"/>
+      <c r="F12" s="25" t="inlineStr"/>
+      <c r="G12" s="25" t="inlineStr"/>
+      <c r="H12" s="25" t="inlineStr"/>
+      <c r="I12" s="25" t="inlineStr"/>
+      <c r="J12" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="L12" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="M12" s="25" t="inlineStr"/>
+      <c r="N12" s="25" t="inlineStr"/>
+      <c r="O12" s="25" t="inlineStr"/>
+      <c r="P12" s="27" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="22" t="inlineStr"/>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 라이브커머스 확산 광고</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>쇼피 라이브 + TikTok Live 연동 / 전환 극대화</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr"/>
+      <c r="E13" s="25" t="inlineStr"/>
+      <c r="F13" s="25" t="inlineStr"/>
+      <c r="G13" s="25" t="inlineStr"/>
+      <c r="H13" s="25" t="inlineStr"/>
+      <c r="I13" s="25" t="inlineStr"/>
+      <c r="J13" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="N13" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="O13" s="25" t="inlineStr"/>
+      <c r="P13" s="27" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>베트남</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr"/>
-      <c r="D12" s="18" t="inlineStr"/>
-      <c r="E12" s="18" t="inlineStr"/>
-      <c r="F12" s="18" t="inlineStr"/>
-      <c r="G12" s="18" t="inlineStr"/>
-      <c r="H12" s="18" t="inlineStr"/>
-      <c r="I12" s="18" t="n">
+      <c r="C14" s="17" t="inlineStr"/>
+      <c r="D14" s="18" t="inlineStr"/>
+      <c r="E14" s="18" t="inlineStr"/>
+      <c r="F14" s="18" t="inlineStr"/>
+      <c r="G14" s="18" t="inlineStr"/>
+      <c r="H14" s="18" t="inlineStr"/>
+      <c r="I14" s="18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>130</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>170</v>
+      </c>
+      <c r="L14" s="18" t="n">
+        <v>120</v>
+      </c>
+      <c r="M14" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="18" t="n">
-        <v>75</v>
-      </c>
-      <c r="K12" s="18" t="n">
-        <v>150</v>
-      </c>
-      <c r="L12" s="18" t="n">
-        <v>55</v>
-      </c>
-      <c r="M12" s="18" t="n">
-        <v>100</v>
-      </c>
-      <c r="N12" s="18" t="n">
-        <v>40</v>
-      </c>
-      <c r="O12" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P12" s="19" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="N14" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="O14" s="18" t="inlineStr"/>
+      <c r="P14" s="19" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>일본</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 코스트코 데모 행사 효율 향상 + 뉴케어 지속 운영 |  6/5 활동 시작</t>
         </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="31" t="inlineStr"/>
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 인플루언서 마케팅 (인스타+광고코드+현장스케치 영상)</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>행사 알림+브랜드 노출 / 6월 집중 런칭</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr"/>
-      <c r="E14" s="25" t="inlineStr"/>
-      <c r="F14" s="25" t="inlineStr"/>
-      <c r="G14" s="25" t="inlineStr"/>
-      <c r="H14" s="25" t="inlineStr"/>
-      <c r="I14" s="34" t="n">
-        <v>25</v>
-      </c>
-      <c r="J14" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="K14" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="L14" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="M14" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="N14" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="O14" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="P14" s="35" t="n">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="31" t="inlineStr"/>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 뉴케어 일본 인스타 브랜드페이지 + 체험단</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>월 5백만 고정 운영 / 리뷰 콘텐츠 누적</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="inlineStr"/>
-      <c r="E15" s="25" t="inlineStr"/>
-      <c r="F15" s="25" t="inlineStr"/>
-      <c r="G15" s="25" t="inlineStr"/>
-      <c r="H15" s="25" t="inlineStr"/>
-      <c r="I15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="J15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="L15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="M15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="N15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="O15" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="P15" s="35" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="31" t="inlineStr"/>
       <c r="B16" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 칼비 후루그라 코스트코 공동 샘플링 협업</t>
+          <t xml:space="preserve"> 인플루언서 마케팅 (인스타+광고코드+현장스케치 영상)</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>후루그라 검색→웰라이프 유입 전략</t>
+          <t>행사 알림+브랜드 노출 / 6월 집중 런칭</t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr"/>
@@ -1683,28 +1667,38 @@
       <c r="I16" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="J16" s="25" t="inlineStr"/>
-      <c r="K16" s="25" t="inlineStr"/>
+      <c r="J16" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="K16" s="34" t="n">
+        <v>15</v>
+      </c>
       <c r="L16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="M16" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="M16" s="25" t="inlineStr"/>
-      <c r="N16" s="25" t="inlineStr"/>
-      <c r="O16" s="25" t="inlineStr"/>
+      <c r="N16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="O16" s="34" t="n">
+        <v>5</v>
+      </c>
       <c r="P16" s="35" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="31" t="inlineStr"/>
       <c r="B17" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 홈쇼핑/라이브커머스/온라인 오픈 SA·DA</t>
+          <t xml:space="preserve"> 뉴케어 일본 인스타 브랜드페이지 + 체험단</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>오픈 시점 집중 광고 집행</t>
+          <t>월 5백만 고정 운영 / 리뷰 콘텐츠 누적</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr"/>
@@ -1712,153 +1706,157 @@
       <c r="F17" s="25" t="inlineStr"/>
       <c r="G17" s="25" t="inlineStr"/>
       <c r="H17" s="25" t="inlineStr"/>
-      <c r="I17" s="25" t="inlineStr"/>
+      <c r="I17" s="34" t="n">
+        <v>5</v>
+      </c>
       <c r="J17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="M17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="N17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="P17" s="35" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="31" t="inlineStr"/>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 칼비 후루그라 코스트코 공동 샘플링 협업</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>후루그라 검색→웰라이프 유입 / 레시피 콘텐츠 연계</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr"/>
+      <c r="E18" s="25" t="inlineStr"/>
+      <c r="F18" s="25" t="inlineStr"/>
+      <c r="G18" s="25" t="inlineStr"/>
+      <c r="H18" s="25" t="inlineStr"/>
+      <c r="I18" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K17" s="25" t="inlineStr"/>
-      <c r="L17" s="25" t="inlineStr"/>
-      <c r="M17" s="25" t="inlineStr"/>
-      <c r="N17" s="34" t="n">
+      <c r="J18" s="25" t="inlineStr"/>
+      <c r="K18" s="25" t="inlineStr"/>
+      <c r="L18" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="M18" s="25" t="inlineStr"/>
+      <c r="N18" s="25" t="inlineStr"/>
+      <c r="O18" s="25" t="inlineStr"/>
+      <c r="P18" s="35" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="31" t="inlineStr"/>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 홈쇼핑/라이브커머스/온라인 오픈 SA·DA</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>오픈 시점 집중 광고 집행</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr"/>
+      <c r="E19" s="25" t="inlineStr"/>
+      <c r="F19" s="25" t="inlineStr"/>
+      <c r="G19" s="25" t="inlineStr"/>
+      <c r="H19" s="25" t="inlineStr"/>
+      <c r="I19" s="25" t="inlineStr"/>
+      <c r="J19" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="O17" s="25" t="inlineStr"/>
-      <c r="P17" s="35" t="n">
+      <c r="K19" s="25" t="inlineStr"/>
+      <c r="L19" s="25" t="inlineStr"/>
+      <c r="M19" s="25" t="inlineStr"/>
+      <c r="N19" s="25" t="inlineStr"/>
+      <c r="O19" s="25" t="inlineStr"/>
+      <c r="P19" s="35" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>소계</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr"/>
+      <c r="D20" s="18" t="inlineStr"/>
+      <c r="E20" s="18" t="inlineStr"/>
+      <c r="F20" s="18" t="inlineStr"/>
+      <c r="G20" s="18" t="inlineStr"/>
+      <c r="H20" s="18" t="inlineStr"/>
+      <c r="I20" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="J20" s="18" t="n">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="36" t="inlineStr">
-        <is>
-          <t>일본</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>소계</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr"/>
-      <c r="D18" s="18" t="inlineStr"/>
-      <c r="E18" s="18" t="inlineStr"/>
-      <c r="F18" s="18" t="inlineStr"/>
-      <c r="G18" s="18" t="inlineStr"/>
-      <c r="H18" s="18" t="inlineStr"/>
-      <c r="I18" s="18" t="n">
-        <v>50</v>
-      </c>
-      <c r="J18" s="18" t="n">
-        <v>45</v>
-      </c>
-      <c r="K18" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="L18" s="18" t="n">
-        <v>35</v>
-      </c>
-      <c r="M18" s="18" t="n">
+      <c r="K20" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="N18" s="18" t="n">
-        <v>35</v>
-      </c>
-      <c r="O18" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P18" s="19" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="L20" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="M20" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="N20" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="O20" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P20" s="19" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 시장진입 초기 인지도·주의 확보 | 대상아메리카 협업 예정</t>
         </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="39" t="inlineStr"/>
-      <c r="B20" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 브랜드 전용존 구축 + 현장 시음 진행</t>
-        </is>
-      </c>
-      <c r="C20" s="41" t="inlineStr">
-        <is>
-          <t>매대 전용 섹션 세팅 + 시음 에이전시</t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="inlineStr"/>
-      <c r="E20" s="25" t="inlineStr"/>
-      <c r="F20" s="25" t="inlineStr"/>
-      <c r="G20" s="25" t="inlineStr"/>
-      <c r="H20" s="25" t="inlineStr"/>
-      <c r="I20" s="42" t="n">
-        <v>25</v>
-      </c>
-      <c r="J20" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="K20" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L20" s="25" t="inlineStr"/>
-      <c r="M20" s="25" t="inlineStr"/>
-      <c r="N20" s="25" t="inlineStr"/>
-      <c r="O20" s="25" t="inlineStr"/>
-      <c r="P20" s="43" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="39" t="inlineStr"/>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>️ 블랙프라이데이·Cyber Monday 이벤트</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="inlineStr">
-        <is>
-          <t>10월 준비 / 11월 집중 집행</t>
-        </is>
-      </c>
-      <c r="D21" s="25" t="inlineStr"/>
-      <c r="E21" s="25" t="inlineStr"/>
-      <c r="F21" s="25" t="inlineStr"/>
-      <c r="G21" s="25" t="inlineStr"/>
-      <c r="H21" s="25" t="inlineStr"/>
-      <c r="I21" s="25" t="inlineStr"/>
-      <c r="J21" s="25" t="inlineStr"/>
-      <c r="K21" s="25" t="inlineStr"/>
-      <c r="L21" s="25" t="inlineStr"/>
-      <c r="M21" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="N21" s="42" t="n">
-        <v>40</v>
-      </c>
-      <c r="O21" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="P21" s="43" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="39" t="inlineStr"/>
       <c r="B22" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 헤이N 브랜드 아마존 테스트 광고</t>
+          <t xml:space="preserve"> 브랜드 전용존 구축 + 현장 시음 진행</t>
         </is>
       </c>
       <c r="C22" s="41" t="inlineStr">
         <is>
-          <t>아마존 Sponsored·PPC 테스트 집행</t>
+          <t>매대 전용 섹션 세팅 + 시음 에이전시</t>
         </is>
       </c>
       <c r="D22" s="25" t="inlineStr"/>
@@ -1866,159 +1864,161 @@
       <c r="F22" s="25" t="inlineStr"/>
       <c r="G22" s="25" t="inlineStr"/>
       <c r="H22" s="25" t="inlineStr"/>
-      <c r="I22" s="25" t="inlineStr"/>
+      <c r="I22" s="42" t="n">
+        <v>25</v>
+      </c>
       <c r="J22" s="42" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K22" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="L22" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="M22" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="N22" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="O22" s="42" t="n">
-        <v>5</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="L22" s="25" t="inlineStr"/>
+      <c r="M22" s="25" t="inlineStr"/>
+      <c r="N22" s="25" t="inlineStr"/>
+      <c r="O22" s="25" t="inlineStr"/>
       <c r="P22" s="43" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="44" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr"/>
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>️ 블랙프라이데이·Cyber Monday 이벤트</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>10월 준비 / 11월 집중 집행</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr"/>
+      <c r="E23" s="25" t="inlineStr"/>
+      <c r="F23" s="25" t="inlineStr"/>
+      <c r="G23" s="25" t="inlineStr"/>
+      <c r="H23" s="25" t="inlineStr"/>
+      <c r="I23" s="25" t="inlineStr"/>
+      <c r="J23" s="25" t="inlineStr"/>
+      <c r="K23" s="25" t="inlineStr"/>
+      <c r="L23" s="25" t="inlineStr"/>
+      <c r="M23" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" s="42" t="n">
+        <v>40</v>
+      </c>
+      <c r="O23" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="P23" s="43" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="39" t="inlineStr"/>
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 헤이N 브랜드 아마존 테스트 광고</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>아마존 Sponsored·PPC 테스트 집행</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="inlineStr"/>
+      <c r="E24" s="25" t="inlineStr"/>
+      <c r="F24" s="25" t="inlineStr"/>
+      <c r="G24" s="25" t="inlineStr"/>
+      <c r="H24" s="25" t="inlineStr"/>
+      <c r="I24" s="25" t="inlineStr"/>
+      <c r="J24" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="K24" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="L24" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="M24" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="N24" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="O24" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="P24" s="43" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="44" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr"/>
-      <c r="D23" s="18" t="inlineStr"/>
-      <c r="E23" s="18" t="inlineStr"/>
-      <c r="F23" s="18" t="inlineStr"/>
-      <c r="G23" s="18" t="inlineStr"/>
-      <c r="H23" s="18" t="inlineStr"/>
-      <c r="I23" s="18" t="n">
+      <c r="C25" s="17" t="inlineStr"/>
+      <c r="D25" s="18" t="inlineStr"/>
+      <c r="E25" s="18" t="inlineStr"/>
+      <c r="F25" s="18" t="inlineStr"/>
+      <c r="G25" s="18" t="inlineStr"/>
+      <c r="H25" s="18" t="inlineStr"/>
+      <c r="I25" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="J23" s="18" t="n">
+      <c r="J25" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K23" s="18" t="n">
+      <c r="K25" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="L23" s="18" t="n">
+      <c r="L25" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="M23" s="18" t="n">
+      <c r="M25" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="N23" s="18" t="n">
+      <c r="N25" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="O23" s="18" t="n">
+      <c r="O25" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="P23" s="19" t="n">
+      <c r="P25" s="19" t="n">
         <v>160</v>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="45" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="45" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="B24" s="46" t="inlineStr">
+      <c r="B26" s="46" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 역직구 채널 안정화 + GP Top5 진입 | 화룬강중 신규 800 파이프라인 런칭</t>
         </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="47" t="inlineStr"/>
-      <c r="B25" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
-        </is>
-      </c>
-      <c r="C25" s="49" t="inlineStr">
-        <is>
-          <t>6/18 D-day 집중 집행</t>
-        </is>
-      </c>
-      <c r="D25" s="25" t="inlineStr"/>
-      <c r="E25" s="25" t="inlineStr"/>
-      <c r="F25" s="25" t="inlineStr"/>
-      <c r="G25" s="25" t="inlineStr"/>
-      <c r="H25" s="25" t="inlineStr"/>
-      <c r="I25" s="50" t="n">
-        <v>60</v>
-      </c>
-      <c r="J25" s="25" t="inlineStr"/>
-      <c r="K25" s="25" t="inlineStr"/>
-      <c r="L25" s="25" t="inlineStr"/>
-      <c r="M25" s="25" t="inlineStr"/>
-      <c r="N25" s="25" t="inlineStr"/>
-      <c r="O25" s="25" t="inlineStr"/>
-      <c r="P25" s="51" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="47" t="inlineStr"/>
-      <c r="B26" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
-        </is>
-      </c>
-      <c r="C26" s="49" t="inlineStr">
-        <is>
-          <t>7~10월 KOL 주기 배포</t>
-        </is>
-      </c>
-      <c r="D26" s="25" t="inlineStr"/>
-      <c r="E26" s="25" t="inlineStr"/>
-      <c r="F26" s="25" t="inlineStr"/>
-      <c r="G26" s="25" t="inlineStr"/>
-      <c r="H26" s="25" t="inlineStr"/>
-      <c r="I26" s="25" t="inlineStr"/>
-      <c r="J26" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="K26" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="L26" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="M26" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="N26" s="25" t="inlineStr"/>
-      <c r="O26" s="25" t="inlineStr"/>
-      <c r="P26" s="51" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="47" t="inlineStr"/>
       <c r="B27" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 광군절 11.11 집중 캠페인</t>
+          <t xml:space="preserve"> 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
         </is>
       </c>
       <c r="C27" s="49" t="inlineStr">
         <is>
-          <t>10월 예열 + 11월 D-day</t>
+          <t>6/18 D-day 집중 집행</t>
         </is>
       </c>
       <c r="D27" s="25" t="inlineStr"/>
@@ -2026,31 +2026,29 @@
       <c r="F27" s="25" t="inlineStr"/>
       <c r="G27" s="25" t="inlineStr"/>
       <c r="H27" s="25" t="inlineStr"/>
-      <c r="I27" s="25" t="inlineStr"/>
+      <c r="I27" s="50" t="n">
+        <v>60</v>
+      </c>
       <c r="J27" s="25" t="inlineStr"/>
       <c r="K27" s="25" t="inlineStr"/>
       <c r="L27" s="25" t="inlineStr"/>
-      <c r="M27" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="N27" s="50" t="n">
-        <v>60</v>
-      </c>
+      <c r="M27" s="25" t="inlineStr"/>
+      <c r="N27" s="25" t="inlineStr"/>
       <c r="O27" s="25" t="inlineStr"/>
       <c r="P27" s="51" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="47" t="inlineStr"/>
       <c r="B28" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 쌍12 (12/12) 연말 마감 캠페인</t>
+          <t xml:space="preserve"> KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
         </is>
       </c>
       <c r="C28" s="49" t="inlineStr">
         <is>
-          <t>연간 목표 달성 마감</t>
+          <t>7~10월 KOL 주기 배포</t>
         </is>
       </c>
       <c r="D28" s="25" t="inlineStr"/>
@@ -2059,28 +2057,34 @@
       <c r="G28" s="25" t="inlineStr"/>
       <c r="H28" s="25" t="inlineStr"/>
       <c r="I28" s="25" t="inlineStr"/>
-      <c r="J28" s="25" t="inlineStr"/>
-      <c r="K28" s="25" t="inlineStr"/>
-      <c r="L28" s="25" t="inlineStr"/>
-      <c r="M28" s="25" t="inlineStr"/>
+      <c r="J28" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="K28" s="50" t="n">
+        <v>25</v>
+      </c>
+      <c r="L28" s="50" t="n">
+        <v>25</v>
+      </c>
+      <c r="M28" s="50" t="n">
+        <v>10</v>
+      </c>
       <c r="N28" s="25" t="inlineStr"/>
-      <c r="O28" s="50" t="n">
-        <v>30</v>
-      </c>
+      <c r="O28" s="25" t="inlineStr"/>
       <c r="P28" s="51" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="47" t="inlineStr"/>
       <c r="B29" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 화룬강중 (신규) 런칭 지원</t>
+          <t xml:space="preserve"> 광군절 11.11 집중 캠페인</t>
         </is>
       </c>
       <c r="C29" s="49" t="inlineStr">
         <is>
-          <t>800 파이프라인 / 런칭 예산 우선 배정 / 케이코스메몰 축소분 재배분</t>
+          <t>10월 예열 + 11월 D-day</t>
         </is>
       </c>
       <c r="D29" s="25" t="inlineStr"/>
@@ -2088,635 +2092,649 @@
       <c r="F29" s="25" t="inlineStr"/>
       <c r="G29" s="25" t="inlineStr"/>
       <c r="H29" s="25" t="inlineStr"/>
-      <c r="I29" s="50" t="n">
+      <c r="I29" s="25" t="inlineStr"/>
+      <c r="J29" s="25" t="inlineStr"/>
+      <c r="K29" s="25" t="inlineStr"/>
+      <c r="L29" s="25" t="inlineStr"/>
+      <c r="M29" s="50" t="n">
         <v>20</v>
       </c>
-      <c r="J29" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="K29" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="L29" s="25" t="inlineStr"/>
-      <c r="M29" s="25" t="inlineStr"/>
-      <c r="N29" s="25" t="inlineStr"/>
+      <c r="N29" s="50" t="n">
+        <v>60</v>
+      </c>
       <c r="O29" s="25" t="inlineStr"/>
       <c r="P29" s="51" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="52" t="inlineStr">
+      <c r="A30" s="47" t="inlineStr"/>
+      <c r="B30" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 쌍12 (12/12) 연말 마감 캠페인</t>
+        </is>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>연간 목표 달성 마감</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="inlineStr"/>
+      <c r="E30" s="25" t="inlineStr"/>
+      <c r="F30" s="25" t="inlineStr"/>
+      <c r="G30" s="25" t="inlineStr"/>
+      <c r="H30" s="25" t="inlineStr"/>
+      <c r="I30" s="25" t="inlineStr"/>
+      <c r="J30" s="25" t="inlineStr"/>
+      <c r="K30" s="25" t="inlineStr"/>
+      <c r="L30" s="25" t="inlineStr"/>
+      <c r="M30" s="25" t="inlineStr"/>
+      <c r="N30" s="25" t="inlineStr"/>
+      <c r="O30" s="50" t="n">
+        <v>30</v>
+      </c>
+      <c r="P30" s="51" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="47" t="inlineStr"/>
+      <c r="B31" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 화룬강중 (신규) 런칭 지원</t>
+        </is>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>800 파이프라인 / 런칭 예산 우선 배정 / 케이코스메몰 축소분 재배분</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr"/>
+      <c r="E31" s="25" t="inlineStr"/>
+      <c r="F31" s="25" t="inlineStr"/>
+      <c r="G31" s="25" t="inlineStr"/>
+      <c r="H31" s="25" t="inlineStr"/>
+      <c r="I31" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="J31" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="K31" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="L31" s="25" t="inlineStr"/>
+      <c r="M31" s="25" t="inlineStr"/>
+      <c r="N31" s="25" t="inlineStr"/>
+      <c r="O31" s="25" t="inlineStr"/>
+      <c r="P31" s="51" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="52" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr"/>
-      <c r="D30" s="18" t="inlineStr"/>
-      <c r="E30" s="18" t="inlineStr"/>
-      <c r="F30" s="18" t="inlineStr"/>
-      <c r="G30" s="18" t="inlineStr"/>
-      <c r="H30" s="18" t="inlineStr"/>
-      <c r="I30" s="18" t="n">
-        <v>80</v>
-      </c>
-      <c r="J30" s="18" t="n">
+      <c r="C32" s="17" t="inlineStr"/>
+      <c r="D32" s="18" t="inlineStr"/>
+      <c r="E32" s="18" t="inlineStr"/>
+      <c r="F32" s="18" t="inlineStr"/>
+      <c r="G32" s="18" t="inlineStr"/>
+      <c r="H32" s="18" t="inlineStr"/>
+      <c r="I32" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="J32" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="K32" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="K30" s="18" t="n">
-        <v>35</v>
-      </c>
-      <c r="L30" s="18" t="n">
+      <c r="L32" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="M30" s="18" t="n">
+      <c r="M32" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="N30" s="18" t="n">
+      <c r="N32" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="O30" s="18" t="n">
+      <c r="O32" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="P30" s="19" t="n">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="P32" s="19" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>대만</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 음료시장 성수기 집중 + Medfirst FSMP Top3 달성</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="53" t="inlineStr"/>
-      <c r="B32" s="54" t="inlineStr">
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 음료시장 성수기 집중 + Medfirst GP Top3 달성</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="53" t="inlineStr"/>
+      <c r="B34" s="54" t="inlineStr">
         <is>
           <t>️ 여름 음료 성수기 집중 광고 (7~9월)</t>
         </is>
       </c>
-      <c r="C32" s="55" t="inlineStr">
+      <c r="C34" s="55" t="inlineStr">
         <is>
           <t>여름 건강음료 수요 피크 시즌</t>
         </is>
       </c>
-      <c r="D32" s="25" t="inlineStr"/>
-      <c r="E32" s="25" t="inlineStr"/>
-      <c r="F32" s="25" t="inlineStr"/>
-      <c r="G32" s="25" t="inlineStr"/>
-      <c r="H32" s="25" t="inlineStr"/>
-      <c r="I32" s="25" t="inlineStr"/>
-      <c r="J32" s="56" t="n">
+      <c r="D34" s="25" t="inlineStr"/>
+      <c r="E34" s="25" t="inlineStr"/>
+      <c r="F34" s="25" t="inlineStr"/>
+      <c r="G34" s="25" t="inlineStr"/>
+      <c r="H34" s="25" t="inlineStr"/>
+      <c r="I34" s="25" t="inlineStr"/>
+      <c r="J34" s="56" t="n">
         <v>20</v>
       </c>
-      <c r="K32" s="56" t="n">
+      <c r="K34" s="56" t="n">
         <v>25</v>
       </c>
-      <c r="L32" s="56" t="n">
+      <c r="L34" s="56" t="n">
         <v>15</v>
       </c>
-      <c r="M32" s="25" t="inlineStr"/>
-      <c r="N32" s="25" t="inlineStr"/>
-      <c r="O32" s="25" t="inlineStr"/>
-      <c r="P32" s="57" t="n">
+      <c r="M34" s="25" t="inlineStr"/>
+      <c r="N34" s="25" t="inlineStr"/>
+      <c r="O34" s="25" t="inlineStr"/>
+      <c r="P34" s="57" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="53" t="inlineStr"/>
-      <c r="B33" s="54" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="53" t="inlineStr"/>
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve"> Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
         </is>
       </c>
-      <c r="C33" s="55" t="inlineStr">
+      <c r="C35" s="55" t="inlineStr">
         <is>
           <t>닥터 추천 마크 부착 후 집행</t>
         </is>
       </c>
-      <c r="D33" s="25" t="inlineStr"/>
-      <c r="E33" s="25" t="inlineStr"/>
-      <c r="F33" s="25" t="inlineStr"/>
-      <c r="G33" s="25" t="inlineStr"/>
-      <c r="H33" s="25" t="inlineStr"/>
-      <c r="I33" s="25" t="inlineStr"/>
-      <c r="J33" s="25" t="inlineStr"/>
-      <c r="K33" s="25" t="inlineStr"/>
-      <c r="L33" s="25" t="inlineStr"/>
-      <c r="M33" s="56" t="n">
-        <v>10</v>
-      </c>
-      <c r="N33" s="25" t="inlineStr"/>
-      <c r="O33" s="56" t="n">
-        <v>10</v>
-      </c>
-      <c r="P33" s="57" t="n">
+      <c r="D35" s="25" t="inlineStr"/>
+      <c r="E35" s="25" t="inlineStr"/>
+      <c r="F35" s="25" t="inlineStr"/>
+      <c r="G35" s="25" t="inlineStr"/>
+      <c r="H35" s="25" t="inlineStr"/>
+      <c r="I35" s="25" t="inlineStr"/>
+      <c r="J35" s="25" t="inlineStr"/>
+      <c r="K35" s="25" t="inlineStr"/>
+      <c r="L35" s="25" t="inlineStr"/>
+      <c r="M35" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="N35" s="25" t="inlineStr"/>
+      <c r="O35" s="25" t="inlineStr"/>
+      <c r="P35" s="57" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>대만</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>소계</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr"/>
+      <c r="D36" s="18" t="inlineStr"/>
+      <c r="E36" s="18" t="inlineStr"/>
+      <c r="F36" s="18" t="inlineStr"/>
+      <c r="G36" s="18" t="inlineStr"/>
+      <c r="H36" s="18" t="inlineStr"/>
+      <c r="I36" s="18" t="inlineStr"/>
+      <c r="J36" s="18" t="n">
         <v>20</v>
       </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t>대만</t>
-        </is>
-      </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="K36" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="L36" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="M36" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="N36" s="18" t="inlineStr"/>
+      <c r="O36" s="18" t="inlineStr"/>
+      <c r="P36" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="58" t="inlineStr">
+        <is>
+          <t>몽골</t>
+        </is>
+      </c>
+      <c r="B37" s="59" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 현지 자체 브랜딩 지원 + 스포츠 마케팅 강화 | 베트남 골든 없음 → 인서트 영상 지원 전환</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="60" t="inlineStr"/>
+      <c r="B38" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
+        </is>
+      </c>
+      <c r="C38" s="62" t="inlineStr">
+        <is>
+          <t>현지 파트너 주도 / 웰라이프 지원</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr"/>
+      <c r="E38" s="25" t="inlineStr"/>
+      <c r="F38" s="25" t="inlineStr"/>
+      <c r="G38" s="25" t="inlineStr"/>
+      <c r="H38" s="25" t="inlineStr"/>
+      <c r="I38" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" s="25" t="inlineStr"/>
+      <c r="K38" s="25" t="inlineStr"/>
+      <c r="L38" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="M38" s="25" t="inlineStr"/>
+      <c r="N38" s="25" t="inlineStr"/>
+      <c r="O38" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="P38" s="64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="60" t="inlineStr"/>
+      <c r="B39" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 인서트 영상 제작 + 현지 배포 지원</t>
+        </is>
+      </c>
+      <c r="C39" s="62" t="inlineStr">
+        <is>
+          <t>베트남 골든 채널 종료 → 몽골 자체 SNS 인서트로 전환</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr"/>
+      <c r="E39" s="25" t="inlineStr"/>
+      <c r="F39" s="25" t="inlineStr"/>
+      <c r="G39" s="25" t="inlineStr"/>
+      <c r="H39" s="25" t="inlineStr"/>
+      <c r="I39" s="25" t="inlineStr"/>
+      <c r="J39" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="K39" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="L39" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="M39" s="25" t="inlineStr"/>
+      <c r="N39" s="25" t="inlineStr"/>
+      <c r="O39" s="25" t="inlineStr"/>
+      <c r="P39" s="64" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="65" t="inlineStr">
+        <is>
+          <t>몽골</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr"/>
-      <c r="D34" s="18" t="inlineStr"/>
-      <c r="E34" s="18" t="inlineStr"/>
-      <c r="F34" s="18" t="inlineStr"/>
-      <c r="G34" s="18" t="inlineStr"/>
-      <c r="H34" s="18" t="inlineStr"/>
-      <c r="I34" s="18" t="inlineStr"/>
-      <c r="J34" s="18" t="n">
+      <c r="C40" s="17" t="inlineStr"/>
+      <c r="D40" s="18" t="inlineStr"/>
+      <c r="E40" s="18" t="inlineStr"/>
+      <c r="F40" s="18" t="inlineStr"/>
+      <c r="G40" s="18" t="inlineStr"/>
+      <c r="H40" s="18" t="inlineStr"/>
+      <c r="I40" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K34" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="L34" s="18" t="n">
+      <c r="K40" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="L40" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="M34" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="N34" s="18" t="inlineStr"/>
-      <c r="O34" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P34" s="19" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="58" t="inlineStr">
-        <is>
-          <t>몽골</t>
-        </is>
-      </c>
-      <c r="B35" s="59" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 현지 자체 브랜딩 지원 + 스포츠 마케팅 강화 | 베트남 골든 없음 → 인서트 영상 지원 전환</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="60" t="inlineStr"/>
-      <c r="B36" s="61" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
-        </is>
-      </c>
-      <c r="C36" s="62" t="inlineStr">
-        <is>
-          <t>현지 파트너 주도 / 웰라이프 지원</t>
-        </is>
-      </c>
-      <c r="D36" s="25" t="inlineStr"/>
-      <c r="E36" s="25" t="inlineStr"/>
-      <c r="F36" s="25" t="inlineStr"/>
-      <c r="G36" s="25" t="inlineStr"/>
-      <c r="H36" s="25" t="inlineStr"/>
-      <c r="I36" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="J36" s="25" t="inlineStr"/>
-      <c r="K36" s="25" t="inlineStr"/>
-      <c r="L36" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="M36" s="25" t="inlineStr"/>
-      <c r="N36" s="25" t="inlineStr"/>
-      <c r="O36" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="P36" s="64" t="n">
+      <c r="M40" s="18" t="inlineStr"/>
+      <c r="N40" s="18" t="inlineStr"/>
+      <c r="O40" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P40" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="58" t="inlineStr">
+        <is>
+          <t>싱가포르</t>
+        </is>
+      </c>
+      <c r="B41" s="59" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 가디언 입점 매출 확대 + EXACTITUDE 리오더 촉진</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="66" t="inlineStr"/>
+      <c r="B42" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 가디언 협업 확대 + 입점 지원</t>
+        </is>
+      </c>
+      <c r="C42" s="68" t="inlineStr">
+        <is>
+          <t>가디언 83개점 확장 / EXACTITUDE 샘플링+판촉 집중</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="inlineStr"/>
+      <c r="E42" s="25" t="inlineStr"/>
+      <c r="F42" s="25" t="inlineStr"/>
+      <c r="G42" s="25" t="inlineStr"/>
+      <c r="H42" s="25" t="inlineStr"/>
+      <c r="I42" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="J42" s="25" t="inlineStr"/>
+      <c r="K42" s="25" t="inlineStr"/>
+      <c r="L42" s="25" t="inlineStr"/>
+      <c r="M42" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="N42" s="25" t="inlineStr"/>
+      <c r="O42" s="25" t="inlineStr"/>
+      <c r="P42" s="70" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="60" t="inlineStr"/>
-      <c r="B37" s="61" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 인서트 영상 제작 + 현지 배포 지원</t>
-        </is>
-      </c>
-      <c r="C37" s="62" t="inlineStr">
-        <is>
-          <t>베트남 골든 채널 종료 → 몽골 자체 SNS 인서트로 전환</t>
-        </is>
-      </c>
-      <c r="D37" s="25" t="inlineStr"/>
-      <c r="E37" s="25" t="inlineStr"/>
-      <c r="F37" s="25" t="inlineStr"/>
-      <c r="G37" s="25" t="inlineStr"/>
-      <c r="H37" s="25" t="inlineStr"/>
-      <c r="I37" s="25" t="inlineStr"/>
-      <c r="J37" s="63" t="n">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="65" t="inlineStr">
+        <is>
+          <t>싱가포르</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>소계</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr"/>
+      <c r="D43" s="18" t="inlineStr"/>
+      <c r="E43" s="18" t="inlineStr"/>
+      <c r="F43" s="18" t="inlineStr"/>
+      <c r="G43" s="18" t="inlineStr"/>
+      <c r="H43" s="18" t="inlineStr"/>
+      <c r="I43" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="J43" s="18" t="inlineStr"/>
+      <c r="K43" s="18" t="inlineStr"/>
+      <c r="L43" s="18" t="inlineStr"/>
+      <c r="M43" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="N43" s="18" t="inlineStr"/>
+      <c r="O43" s="18" t="inlineStr"/>
+      <c r="P43" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="K37" s="63" t="n">
-        <v>20</v>
-      </c>
-      <c r="L37" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="M37" s="25" t="inlineStr"/>
-      <c r="N37" s="25" t="inlineStr"/>
-      <c r="O37" s="25" t="inlineStr"/>
-      <c r="P37" s="64" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="65" t="inlineStr">
-        <is>
-          <t>몽골</t>
-        </is>
-      </c>
-      <c r="B38" s="16" t="inlineStr">
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="71" t="inlineStr">
+        <is>
+          <t>중동</t>
+        </is>
+      </c>
+      <c r="B44" s="72" t="inlineStr">
+        <is>
+          <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="73" t="inlineStr"/>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
+        </is>
+      </c>
+      <c r="C45" s="75" t="inlineStr">
+        <is>
+          <t>현상 유지 / 추가 투자 없음</t>
+        </is>
+      </c>
+      <c r="D45" s="25" t="inlineStr"/>
+      <c r="E45" s="25" t="inlineStr"/>
+      <c r="F45" s="25" t="inlineStr"/>
+      <c r="G45" s="25" t="inlineStr"/>
+      <c r="H45" s="25" t="inlineStr"/>
+      <c r="I45" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="J45" s="25" t="inlineStr"/>
+      <c r="K45" s="25" t="inlineStr"/>
+      <c r="L45" s="25" t="inlineStr"/>
+      <c r="M45" s="25" t="inlineStr"/>
+      <c r="N45" s="25" t="inlineStr"/>
+      <c r="O45" s="25" t="inlineStr"/>
+      <c r="P45" s="77" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="78" t="inlineStr">
+        <is>
+          <t>중동</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr"/>
-      <c r="D38" s="18" t="inlineStr"/>
-      <c r="E38" s="18" t="inlineStr"/>
-      <c r="F38" s="18" t="inlineStr"/>
-      <c r="G38" s="18" t="inlineStr"/>
-      <c r="H38" s="18" t="inlineStr"/>
-      <c r="I38" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J38" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="K38" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="L38" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="M38" s="18" t="inlineStr"/>
-      <c r="N38" s="18" t="inlineStr"/>
-      <c r="O38" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P38" s="19" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="58" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="B39" s="59" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 가디언 입점 매출 확대 + 박람회 신규 채널 개척</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="66" t="inlineStr"/>
-      <c r="B40" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 가디언 협업 확대 + 미팅 후 입점 지원</t>
-        </is>
-      </c>
-      <c r="C40" s="68" t="inlineStr">
-        <is>
-          <t>가디언 83개점 → 확장 공략</t>
-        </is>
-      </c>
-      <c r="D40" s="25" t="inlineStr"/>
-      <c r="E40" s="25" t="inlineStr"/>
-      <c r="F40" s="25" t="inlineStr"/>
-      <c r="G40" s="25" t="inlineStr"/>
-      <c r="H40" s="25" t="inlineStr"/>
-      <c r="I40" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="J40" s="25" t="inlineStr"/>
-      <c r="K40" s="25" t="inlineStr"/>
-      <c r="L40" s="25" t="inlineStr"/>
-      <c r="M40" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="N40" s="25" t="inlineStr"/>
-      <c r="O40" s="25" t="inlineStr"/>
-      <c r="P40" s="70" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="66" t="inlineStr"/>
-      <c r="B41" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 현지 박람회 / 전시회 참가</t>
-        </is>
-      </c>
-      <c r="C41" s="68" t="inlineStr">
-        <is>
-          <t>신규 바이어 발굴</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="inlineStr"/>
-      <c r="E41" s="25" t="inlineStr"/>
-      <c r="F41" s="25" t="inlineStr"/>
-      <c r="G41" s="25" t="inlineStr"/>
-      <c r="H41" s="25" t="inlineStr"/>
-      <c r="I41" s="25" t="inlineStr"/>
-      <c r="J41" s="25" t="inlineStr"/>
-      <c r="K41" s="25" t="inlineStr"/>
-      <c r="L41" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="M41" s="25" t="inlineStr"/>
-      <c r="N41" s="25" t="inlineStr"/>
-      <c r="O41" s="25" t="inlineStr"/>
-      <c r="P41" s="70" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="65" t="inlineStr">
-        <is>
-          <t>싱가포르</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="C46" s="17" t="inlineStr"/>
+      <c r="D46" s="18" t="inlineStr"/>
+      <c r="E46" s="18" t="inlineStr"/>
+      <c r="F46" s="18" t="inlineStr"/>
+      <c r="G46" s="18" t="inlineStr"/>
+      <c r="H46" s="18" t="inlineStr"/>
+      <c r="I46" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J46" s="18" t="inlineStr"/>
+      <c r="K46" s="18" t="inlineStr"/>
+      <c r="L46" s="18" t="inlineStr"/>
+      <c r="M46" s="18" t="inlineStr"/>
+      <c r="N46" s="18" t="inlineStr"/>
+      <c r="O46" s="18" t="inlineStr"/>
+      <c r="P46" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="79" t="inlineStr">
+        <is>
+          <t>호주</t>
+        </is>
+      </c>
+      <c r="B47" s="80" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: 대상 호주 채널 안정화 (천호케어 제외 / 비용대비 성장률 없음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="81" t="inlineStr"/>
+      <c r="B48" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 대상 호주 공동 마케팅 지원</t>
+        </is>
+      </c>
+      <c r="C48" s="83" t="inlineStr">
+        <is>
+          <t>천호케어 제외 / 대상 호주 직접 채널만 지원</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="inlineStr"/>
+      <c r="E48" s="25" t="inlineStr"/>
+      <c r="F48" s="25" t="inlineStr"/>
+      <c r="G48" s="25" t="inlineStr"/>
+      <c r="H48" s="25" t="inlineStr"/>
+      <c r="I48" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="J48" s="25" t="inlineStr"/>
+      <c r="K48" s="25" t="inlineStr"/>
+      <c r="L48" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="M48" s="25" t="inlineStr"/>
+      <c r="N48" s="25" t="inlineStr"/>
+      <c r="O48" s="25" t="inlineStr"/>
+      <c r="P48" s="85" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="86" t="inlineStr">
+        <is>
+          <t>호주</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr"/>
-      <c r="D42" s="18" t="inlineStr"/>
-      <c r="E42" s="18" t="inlineStr"/>
-      <c r="F42" s="18" t="inlineStr"/>
-      <c r="G42" s="18" t="inlineStr"/>
-      <c r="H42" s="18" t="inlineStr"/>
-      <c r="I42" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="J42" s="18" t="inlineStr"/>
-      <c r="K42" s="18" t="inlineStr"/>
-      <c r="L42" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="M42" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="N42" s="18" t="inlineStr"/>
-      <c r="O42" s="18" t="inlineStr"/>
-      <c r="P42" s="19" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="71" t="inlineStr">
-        <is>
-          <t>중동</t>
-        </is>
-      </c>
-      <c r="B43" s="72" t="inlineStr">
-        <is>
-          <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="73" t="inlineStr"/>
-      <c r="B44" s="74" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
-        </is>
-      </c>
-      <c r="C44" s="75" t="inlineStr">
-        <is>
-          <t>현상 유지 / 추가 투자 없음</t>
-        </is>
-      </c>
-      <c r="D44" s="25" t="inlineStr"/>
-      <c r="E44" s="25" t="inlineStr"/>
-      <c r="F44" s="25" t="inlineStr"/>
-      <c r="G44" s="25" t="inlineStr"/>
-      <c r="H44" s="25" t="inlineStr"/>
-      <c r="I44" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="J44" s="25" t="inlineStr"/>
-      <c r="K44" s="25" t="inlineStr"/>
-      <c r="L44" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="M44" s="25" t="inlineStr"/>
-      <c r="N44" s="25" t="inlineStr"/>
-      <c r="O44" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="P44" s="77" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="78" t="inlineStr">
-        <is>
-          <t>중동</t>
-        </is>
-      </c>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>소계</t>
-        </is>
-      </c>
-      <c r="C45" s="17" t="inlineStr"/>
-      <c r="D45" s="18" t="inlineStr"/>
-      <c r="E45" s="18" t="inlineStr"/>
-      <c r="F45" s="18" t="inlineStr"/>
-      <c r="G45" s="18" t="inlineStr"/>
-      <c r="H45" s="18" t="inlineStr"/>
-      <c r="I45" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J45" s="18" t="inlineStr"/>
-      <c r="K45" s="18" t="inlineStr"/>
-      <c r="L45" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="M45" s="18" t="inlineStr"/>
-      <c r="N45" s="18" t="inlineStr"/>
-      <c r="O45" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P45" s="19" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="79" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="B46" s="80" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 천호케어 파트너십 유지 + 대상 호주 채널 안정화</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="81" t="inlineStr"/>
-      <c r="B47" s="82" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 천호케어 + 대상 호주 공동 마케팅 지원</t>
-        </is>
-      </c>
-      <c r="C47" s="83" t="inlineStr">
-        <is>
-          <t>파트너 요청 시 지원</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="inlineStr"/>
-      <c r="E47" s="25" t="inlineStr"/>
-      <c r="F47" s="25" t="inlineStr"/>
-      <c r="G47" s="25" t="inlineStr"/>
-      <c r="H47" s="25" t="inlineStr"/>
-      <c r="I47" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="J47" s="25" t="inlineStr"/>
-      <c r="K47" s="25" t="inlineStr"/>
-      <c r="L47" s="84" t="n">
-        <v>10</v>
-      </c>
-      <c r="M47" s="25" t="inlineStr"/>
-      <c r="N47" s="25" t="inlineStr"/>
-      <c r="O47" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="P47" s="85" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="86" t="inlineStr">
-        <is>
-          <t>호주</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>소계</t>
-        </is>
-      </c>
-      <c r="C48" s="17" t="inlineStr"/>
-      <c r="D48" s="18" t="inlineStr"/>
-      <c r="E48" s="18" t="inlineStr"/>
-      <c r="F48" s="18" t="inlineStr"/>
-      <c r="G48" s="18" t="inlineStr"/>
-      <c r="H48" s="18" t="inlineStr"/>
-      <c r="I48" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J48" s="18" t="inlineStr"/>
-      <c r="K48" s="18" t="inlineStr"/>
-      <c r="L48" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="M48" s="18" t="inlineStr"/>
-      <c r="N48" s="18" t="inlineStr"/>
-      <c r="O48" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="P48" s="19" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="87" t="inlineStr">
+      <c r="C49" s="17" t="inlineStr"/>
+      <c r="D49" s="18" t="inlineStr"/>
+      <c r="E49" s="18" t="inlineStr"/>
+      <c r="F49" s="18" t="inlineStr"/>
+      <c r="G49" s="18" t="inlineStr"/>
+      <c r="H49" s="18" t="inlineStr"/>
+      <c r="I49" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J49" s="18" t="inlineStr"/>
+      <c r="K49" s="18" t="inlineStr"/>
+      <c r="L49" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="M49" s="18" t="inlineStr"/>
+      <c r="N49" s="18" t="inlineStr"/>
+      <c r="O49" s="18" t="inlineStr"/>
+      <c r="P49" s="19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="87" t="inlineStr">
         <is>
           <t>총 합계 (백만원)</t>
         </is>
       </c>
-      <c r="D49" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="E49" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="F49" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="G49" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="H49" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="I49" s="88" t="n">
-        <v>245</v>
-      </c>
-      <c r="J49" s="88" t="n">
-        <v>220</v>
-      </c>
-      <c r="K49" s="88" t="n">
-        <v>290</v>
-      </c>
-      <c r="L49" s="88" t="n">
-        <v>195</v>
-      </c>
-      <c r="M49" s="88" t="n">
-        <v>200</v>
-      </c>
-      <c r="N49" s="88" t="n">
-        <v>190</v>
-      </c>
-      <c r="O49" s="88" t="n">
-        <v>110</v>
-      </c>
-      <c r="P49" s="89" t="n">
+      <c r="D50" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="F50" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="G50" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="H50" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="I50" s="88" t="n">
+        <v>265</v>
+      </c>
+      <c r="J50" s="88" t="n">
+        <v>265</v>
+      </c>
+      <c r="K50" s="88" t="n">
+        <v>300</v>
+      </c>
+      <c r="L50" s="88" t="n">
+        <v>235</v>
+      </c>
+      <c r="M50" s="88" t="n">
+        <v>145</v>
+      </c>
+      <c r="N50" s="88" t="n">
+        <v>165</v>
+      </c>
+      <c r="O50" s="88" t="n">
+        <v>75</v>
+      </c>
+      <c r="P50" s="89" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 295  |  하반기(7~12월) 합계: 1,205  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 315  |  하반기(7~12월) 합계: 1,185  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B43:P43"/>
+    <mergeCell ref="A51:P51"/>
+    <mergeCell ref="B15:P15"/>
     <mergeCell ref="B7:P7"/>
-    <mergeCell ref="B39:P39"/>
-    <mergeCell ref="B24:P24"/>
-    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="B33:P33"/>
+    <mergeCell ref="B44:P44"/>
+    <mergeCell ref="B47:P47"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="B19:P19"/>
-    <mergeCell ref="B31:P31"/>
-    <mergeCell ref="B46:P46"/>
-    <mergeCell ref="A50:P50"/>
-    <mergeCell ref="B35:P35"/>
+    <mergeCell ref="B37:P37"/>
+    <mergeCell ref="B41:P41"/>
     <mergeCell ref="B4:P4"/>
-    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="B26:P26"/>
+    <mergeCell ref="B21:P21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revise all countries: Vietnam CGF 8천만, offline 40stores, Japan 31 influencers+ecobag, Taiwan Medfirst boost
- Vietnam: CGF 논문 6천만+배포 2천만=80M, offline tasting 40stores@25M/mo (6-9월), replace 이너샵VMD with Shopee/Zalo ads, add sampling+live commerce
- Japan: restructure to 31 influencers (test), O2O ecobag event 37stores, ecommerce test, remove 인스타 paid budget (자체운영)
- Taiwan: Medfirst single-channel boost — LINE OA + pharmacist education kit + performance incentive
- Australia: remove 천호케어 (low ROI)
- Total maintained at 1,500M KRW

https://claude.ai/code/session_01FNPFF5mFSuHNsmFNUSkkTX
</commit_message>
<xml_diff>
--- a/2026_글로벌마케팅캘린더.xlsx
+++ b/2026_글로벌마케팅캘린더.xlsx
@@ -1065,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1417,12 +1417,12 @@
       <c r="A9" s="22" t="inlineStr"/>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CGF 전문성 (의사협회 논문 + KOL/KOC)</t>
+          <t xml:space="preserve"> CGF 의사협회 논문 제작</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>6월 논문착수 → 7~10월 KOL/KOC 순차 배포</t>
+          <t>논문 제작비 6,000만 (6월 착수) + 배포·알리기 2,000만</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr"/>
@@ -1431,36 +1431,30 @@
       <c r="G9" s="25" t="inlineStr"/>
       <c r="H9" s="25" t="inlineStr"/>
       <c r="I9" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="J9" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="J9" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="L9" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="M9" s="26" t="n">
-        <v>5</v>
-      </c>
+      <c r="K9" s="25" t="inlineStr"/>
+      <c r="L9" s="25" t="inlineStr"/>
+      <c r="M9" s="25" t="inlineStr"/>
       <c r="N9" s="25" t="inlineStr"/>
       <c r="O9" s="25" t="inlineStr"/>
       <c r="P9" s="27" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="22" t="inlineStr"/>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 오프라인 엔드매대 + 시음행사</t>
+          <t xml:space="preserve"> 오프라인 시음 (롯데/이마트/윈마트 40개점)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>윈마트 262개 확장 / 일본 구조 복사 적용</t>
+          <t>윈마트 15개점 포함 / 월 2,500만 / 6~9월 집중</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr"/>
@@ -1469,38 +1463,34 @@
       <c r="G10" s="25" t="inlineStr"/>
       <c r="H10" s="25" t="inlineStr"/>
       <c r="I10" s="26" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J10" s="26" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="K10" s="26" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="L10" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="M10" s="26" t="n">
-        <v>10</v>
-      </c>
-      <c r="N10" s="26" t="n">
-        <v>10</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="M10" s="25" t="inlineStr"/>
+      <c r="N10" s="25" t="inlineStr"/>
       <c r="O10" s="25" t="inlineStr"/>
       <c r="P10" s="27" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="22" t="inlineStr"/>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 이너샵 VMD + 홍보물 + 온라인</t>
+          <t xml:space="preserve"> 이너샵 대체 — 쇼피Ads + Zalo 타겟광고</t>
         </is>
       </c>
       <c r="C11" s="24" t="inlineStr">
         <is>
-          <t>8월 오픈 연동 / 매장 VMD+SNS 병행</t>
+          <t>이너샵 VMD 대체 / 8월 오픈 연동 / 반경 3km 지오타겟</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr"/>
@@ -1511,7 +1501,7 @@
       <c r="I11" s="25" t="inlineStr"/>
       <c r="J11" s="25" t="inlineStr"/>
       <c r="K11" s="26" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L11" s="26" t="n">
         <v>10</v>
@@ -1520,7 +1510,7 @@
       <c r="N11" s="25" t="inlineStr"/>
       <c r="O11" s="25" t="inlineStr"/>
       <c r="P11" s="27" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -1532,7 +1522,7 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>일본 칼비 구조 복사 / 시음→SNS 후기→재구매 루프</t>
+          <t>시음→SNS 후기→재구매 루프 / 일본 칼비 구조 복사</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr"/>
@@ -1545,7 +1535,7 @@
         <v>10</v>
       </c>
       <c r="K12" s="26" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="L12" s="26" t="n">
         <v>10</v>
@@ -1554,7 +1544,7 @@
       <c r="N12" s="25" t="inlineStr"/>
       <c r="O12" s="25" t="inlineStr"/>
       <c r="P12" s="27" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -1581,18 +1571,12 @@
       <c r="K13" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="L13" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="M13" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="N13" s="26" t="n">
-        <v>5</v>
-      </c>
+      <c r="L13" s="25" t="inlineStr"/>
+      <c r="M13" s="25" t="inlineStr"/>
+      <c r="N13" s="25" t="inlineStr"/>
       <c r="O13" s="25" t="inlineStr"/>
       <c r="P13" s="27" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -1613,26 +1597,26 @@
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="18" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="K14" s="18" t="n">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="L14" s="18" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="M14" s="18" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="N14" s="18" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="O14" s="18" t="inlineStr"/>
       <c r="P14" s="19" t="n">
-        <v>595</v>
+        <v>650</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
@@ -1643,7 +1627,7 @@
       </c>
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t>▶ 목표: 최종목표: 코스트코 데모 행사 효율 향상 + 뉴케어 지속 운영 |  6/5 활동 시작</t>
+          <t>▶ 목표: 최종목표: 코스트코 데모 행사 효율 향상 + 뉴케어 지속 운영 | 6/5 활동 시작 | 인스타 자체운영(비용무)</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1635,12 @@
       <c r="A16" s="31" t="inlineStr"/>
       <c r="B16" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 인플루언서 마케팅 (인스타+광고코드+현장스케치 영상)</t>
+          <t xml:space="preserve"> 인플루언서 마케팅 (31명: 6월 15명/7월 8명/8월 8명)</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>행사 알림+브랜드 노출 / 6월 집중 런칭</t>
+          <t>테스트 후 이후 결정 / 광고코드+현장스케치 영상</t>
         </is>
       </c>
       <c r="D16" s="25" t="inlineStr"/>
@@ -1665,40 +1649,32 @@
       <c r="G16" s="25" t="inlineStr"/>
       <c r="H16" s="25" t="inlineStr"/>
       <c r="I16" s="34" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J16" s="34" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K16" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="L16" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="M16" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="N16" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="O16" s="34" t="n">
-        <v>5</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="L16" s="25" t="inlineStr"/>
+      <c r="M16" s="25" t="inlineStr"/>
+      <c r="N16" s="25" t="inlineStr"/>
+      <c r="O16" s="25" t="inlineStr"/>
       <c r="P16" s="35" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="31" t="inlineStr"/>
       <c r="B17" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 뉴케어 일본 인스타 브랜드페이지 + 체험단</t>
+          <t xml:space="preserve"> O2O 에코백 판촉 이벤트 (37개점 × 50개)</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>월 5백만 고정 운영 / 리뷰 콘텐츠 누적</t>
+          <t>영상 보고 방문자+매장 구입자 에코백 증정 / 개당 2,500원</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr"/>
@@ -1706,41 +1682,29 @@
       <c r="F17" s="25" t="inlineStr"/>
       <c r="G17" s="25" t="inlineStr"/>
       <c r="H17" s="25" t="inlineStr"/>
-      <c r="I17" s="34" t="n">
-        <v>5</v>
-      </c>
+      <c r="I17" s="25" t="inlineStr"/>
       <c r="J17" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="K17" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="N17" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="O17" s="34" t="n">
-        <v>5</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K17" s="25" t="inlineStr"/>
+      <c r="L17" s="25" t="inlineStr"/>
+      <c r="M17" s="25" t="inlineStr"/>
+      <c r="N17" s="25" t="inlineStr"/>
+      <c r="O17" s="25" t="inlineStr"/>
       <c r="P17" s="35" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="31" t="inlineStr"/>
       <c r="B18" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 칼비 후루그라 코스트코 공동 샘플링 협업</t>
+          <t xml:space="preserve"> 이커머스 테스트 (아마존JP / 라쿠텐)</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>후루그라 검색→웰라이프 유입 / 레시피 콘텐츠 연계</t>
+          <t>소규모 Sponsored 테스트 / 전환 데이터 수집</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr"/>
@@ -1748,31 +1712,33 @@
       <c r="F18" s="25" t="inlineStr"/>
       <c r="G18" s="25" t="inlineStr"/>
       <c r="H18" s="25" t="inlineStr"/>
-      <c r="I18" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="J18" s="25" t="inlineStr"/>
-      <c r="K18" s="25" t="inlineStr"/>
+      <c r="I18" s="25" t="inlineStr"/>
+      <c r="J18" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" s="34" t="n">
+        <v>10</v>
+      </c>
       <c r="L18" s="34" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M18" s="25" t="inlineStr"/>
       <c r="N18" s="25" t="inlineStr"/>
       <c r="O18" s="25" t="inlineStr"/>
       <c r="P18" s="35" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="31" t="inlineStr"/>
       <c r="B19" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 홈쇼핑/라이브커머스/온라인 오픈 SA·DA</t>
+          <t xml:space="preserve"> 칼비 후루그라 코스트코 공동 샘플링 협업</t>
         </is>
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>오픈 시점 집중 광고 집행</t>
+          <t>후루그라 검색→웰라이프 유입 / 레시피 콘텐츠 연계</t>
         </is>
       </c>
       <c r="D19" s="25" t="inlineStr"/>
@@ -1780,117 +1746,109 @@
       <c r="F19" s="25" t="inlineStr"/>
       <c r="G19" s="25" t="inlineStr"/>
       <c r="H19" s="25" t="inlineStr"/>
-      <c r="I19" s="25" t="inlineStr"/>
-      <c r="J19" s="34" t="n">
+      <c r="I19" s="34" t="n">
         <v>20</v>
       </c>
+      <c r="J19" s="25" t="inlineStr"/>
       <c r="K19" s="25" t="inlineStr"/>
-      <c r="L19" s="25" t="inlineStr"/>
+      <c r="L19" s="34" t="n">
+        <v>15</v>
+      </c>
       <c r="M19" s="25" t="inlineStr"/>
       <c r="N19" s="25" t="inlineStr"/>
       <c r="O19" s="25" t="inlineStr"/>
       <c r="P19" s="35" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="31" t="inlineStr"/>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 홈쇼핑/라이브커머스 SA·DA</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>오픈 시점 집중 광고 / 7월 집행</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr"/>
+      <c r="E20" s="25" t="inlineStr"/>
+      <c r="F20" s="25" t="inlineStr"/>
+      <c r="G20" s="25" t="inlineStr"/>
+      <c r="H20" s="25" t="inlineStr"/>
+      <c r="I20" s="25" t="inlineStr"/>
+      <c r="J20" s="34" t="n">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="K20" s="25" t="inlineStr"/>
+      <c r="L20" s="25" t="inlineStr"/>
+      <c r="M20" s="25" t="inlineStr"/>
+      <c r="N20" s="25" t="inlineStr"/>
+      <c r="O20" s="25" t="inlineStr"/>
+      <c r="P20" s="35" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>일본</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr"/>
-      <c r="D20" s="18" t="inlineStr"/>
-      <c r="E20" s="18" t="inlineStr"/>
-      <c r="F20" s="18" t="inlineStr"/>
-      <c r="G20" s="18" t="inlineStr"/>
-      <c r="H20" s="18" t="inlineStr"/>
-      <c r="I20" s="18" t="n">
-        <v>45</v>
-      </c>
-      <c r="J20" s="18" t="n">
-        <v>40</v>
-      </c>
-      <c r="K20" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="L20" s="18" t="n">
-        <v>30</v>
-      </c>
-      <c r="M20" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="N20" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="O20" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P20" s="19" t="n">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr"/>
+      <c r="D21" s="18" t="inlineStr"/>
+      <c r="E21" s="18" t="inlineStr"/>
+      <c r="F21" s="18" t="inlineStr"/>
+      <c r="G21" s="18" t="inlineStr"/>
+      <c r="H21" s="18" t="inlineStr"/>
+      <c r="I21" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="J21" s="18" t="n">
+        <v>42</v>
+      </c>
+      <c r="K21" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="L21" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="M21" s="18" t="inlineStr"/>
+      <c r="N21" s="18" t="inlineStr"/>
+      <c r="O21" s="18" t="inlineStr"/>
+      <c r="P21" s="19" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 시장진입 초기 인지도·주의 확보 | 대상아메리카 협업 예정</t>
         </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="39" t="inlineStr"/>
-      <c r="B22" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 브랜드 전용존 구축 + 현장 시음 진행</t>
-        </is>
-      </c>
-      <c r="C22" s="41" t="inlineStr">
-        <is>
-          <t>매대 전용 섹션 세팅 + 시음 에이전시</t>
-        </is>
-      </c>
-      <c r="D22" s="25" t="inlineStr"/>
-      <c r="E22" s="25" t="inlineStr"/>
-      <c r="F22" s="25" t="inlineStr"/>
-      <c r="G22" s="25" t="inlineStr"/>
-      <c r="H22" s="25" t="inlineStr"/>
-      <c r="I22" s="42" t="n">
-        <v>25</v>
-      </c>
-      <c r="J22" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="K22" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L22" s="25" t="inlineStr"/>
-      <c r="M22" s="25" t="inlineStr"/>
-      <c r="N22" s="25" t="inlineStr"/>
-      <c r="O22" s="25" t="inlineStr"/>
-      <c r="P22" s="43" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="39" t="inlineStr"/>
       <c r="B23" s="40" t="inlineStr">
         <is>
-          <t>️ 블랙프라이데이·Cyber Monday 이벤트</t>
+          <t xml:space="preserve"> 브랜드 전용존 구축 + 현장 시음 진행</t>
         </is>
       </c>
       <c r="C23" s="41" t="inlineStr">
         <is>
-          <t>10월 준비 / 11월 집중 집행</t>
+          <t>매대 전용 섹션 세팅 + 시음 에이전시</t>
         </is>
       </c>
       <c r="D23" s="25" t="inlineStr"/>
@@ -1898,33 +1856,33 @@
       <c r="F23" s="25" t="inlineStr"/>
       <c r="G23" s="25" t="inlineStr"/>
       <c r="H23" s="25" t="inlineStr"/>
-      <c r="I23" s="25" t="inlineStr"/>
-      <c r="J23" s="25" t="inlineStr"/>
-      <c r="K23" s="25" t="inlineStr"/>
+      <c r="I23" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J23" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="K23" s="42" t="n">
+        <v>10</v>
+      </c>
       <c r="L23" s="25" t="inlineStr"/>
-      <c r="M23" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="N23" s="42" t="n">
-        <v>40</v>
-      </c>
-      <c r="O23" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="M23" s="25" t="inlineStr"/>
+      <c r="N23" s="25" t="inlineStr"/>
+      <c r="O23" s="25" t="inlineStr"/>
       <c r="P23" s="43" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="39" t="inlineStr"/>
       <c r="B24" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 헤이N 브랜드 아마존 테스트 광고</t>
+          <t>️ 블랙프라이데이·Cyber Monday 이벤트</t>
         </is>
       </c>
       <c r="C24" s="41" t="inlineStr">
         <is>
-          <t>아마존 Sponsored·PPC 테스트 집행</t>
+          <t>10월 준비 / 11월 집중 집행</t>
         </is>
       </c>
       <c r="D24" s="25" t="inlineStr"/>
@@ -1933,122 +1891,126 @@
       <c r="G24" s="25" t="inlineStr"/>
       <c r="H24" s="25" t="inlineStr"/>
       <c r="I24" s="25" t="inlineStr"/>
-      <c r="J24" s="42" t="n">
+      <c r="J24" s="25" t="inlineStr"/>
+      <c r="K24" s="25" t="inlineStr"/>
+      <c r="L24" s="25" t="inlineStr"/>
+      <c r="M24" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" s="42" t="n">
+        <v>40</v>
+      </c>
+      <c r="O24" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="P24" s="43" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="39" t="inlineStr"/>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 헤이N 브랜드 아마존 테스트 광고</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>아마존 Sponsored·PPC 테스트 집행</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="inlineStr"/>
+      <c r="E25" s="25" t="inlineStr"/>
+      <c r="F25" s="25" t="inlineStr"/>
+      <c r="G25" s="25" t="inlineStr"/>
+      <c r="H25" s="25" t="inlineStr"/>
+      <c r="I25" s="25" t="inlineStr"/>
+      <c r="J25" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="K24" s="42" t="n">
+      <c r="K25" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="L24" s="42" t="n">
+      <c r="L25" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="M24" s="42" t="n">
+      <c r="M25" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="N24" s="42" t="n">
+      <c r="N25" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="O24" s="42" t="n">
+      <c r="O25" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="P24" s="43" t="n">
+      <c r="P25" s="43" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="44" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="44" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr"/>
-      <c r="D25" s="18" t="inlineStr"/>
-      <c r="E25" s="18" t="inlineStr"/>
-      <c r="F25" s="18" t="inlineStr"/>
-      <c r="G25" s="18" t="inlineStr"/>
-      <c r="H25" s="18" t="inlineStr"/>
-      <c r="I25" s="18" t="n">
+      <c r="C26" s="17" t="inlineStr"/>
+      <c r="D26" s="18" t="inlineStr"/>
+      <c r="E26" s="18" t="inlineStr"/>
+      <c r="F26" s="18" t="inlineStr"/>
+      <c r="G26" s="18" t="inlineStr"/>
+      <c r="H26" s="18" t="inlineStr"/>
+      <c r="I26" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="J25" s="18" t="n">
+      <c r="J26" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K25" s="18" t="n">
+      <c r="K26" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="L25" s="18" t="n">
+      <c r="L26" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="M25" s="18" t="n">
+      <c r="M26" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="N25" s="18" t="n">
+      <c r="N26" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="O25" s="18" t="n">
+      <c r="O26" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="P25" s="19" t="n">
+      <c r="P26" s="19" t="n">
         <v>160</v>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="45" t="inlineStr">
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="45" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="B26" s="46" t="inlineStr">
+      <c r="B27" s="46" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 역직구 채널 안정화 + GP Top5 진입 | 화룬강중 신규 800 파이프라인 런칭</t>
         </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="47" t="inlineStr"/>
-      <c r="B27" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
-        </is>
-      </c>
-      <c r="C27" s="49" t="inlineStr">
-        <is>
-          <t>6/18 D-day 집중 집행</t>
-        </is>
-      </c>
-      <c r="D27" s="25" t="inlineStr"/>
-      <c r="E27" s="25" t="inlineStr"/>
-      <c r="F27" s="25" t="inlineStr"/>
-      <c r="G27" s="25" t="inlineStr"/>
-      <c r="H27" s="25" t="inlineStr"/>
-      <c r="I27" s="50" t="n">
-        <v>60</v>
-      </c>
-      <c r="J27" s="25" t="inlineStr"/>
-      <c r="K27" s="25" t="inlineStr"/>
-      <c r="L27" s="25" t="inlineStr"/>
-      <c r="M27" s="25" t="inlineStr"/>
-      <c r="N27" s="25" t="inlineStr"/>
-      <c r="O27" s="25" t="inlineStr"/>
-      <c r="P27" s="51" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="47" t="inlineStr"/>
       <c r="B28" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
+          <t xml:space="preserve"> 618 쇼핑절 KOL 라이브방송 + 역직구 집중</t>
         </is>
       </c>
       <c r="C28" s="49" t="inlineStr">
         <is>
-          <t>7~10월 KOL 주기 배포</t>
+          <t>6/18 D-day 집중 집행</t>
         </is>
       </c>
       <c r="D28" s="25" t="inlineStr"/>
@@ -2056,35 +2018,29 @@
       <c r="F28" s="25" t="inlineStr"/>
       <c r="G28" s="25" t="inlineStr"/>
       <c r="H28" s="25" t="inlineStr"/>
-      <c r="I28" s="25" t="inlineStr"/>
-      <c r="J28" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="K28" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="L28" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="M28" s="50" t="n">
-        <v>10</v>
-      </c>
+      <c r="I28" s="50" t="n">
+        <v>60</v>
+      </c>
+      <c r="J28" s="25" t="inlineStr"/>
+      <c r="K28" s="25" t="inlineStr"/>
+      <c r="L28" s="25" t="inlineStr"/>
+      <c r="M28" s="25" t="inlineStr"/>
       <c r="N28" s="25" t="inlineStr"/>
       <c r="O28" s="25" t="inlineStr"/>
       <c r="P28" s="51" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="47" t="inlineStr"/>
       <c r="B29" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 광군절 11.11 집중 캠페인</t>
+          <t xml:space="preserve"> KOL 영상마케팅 + 전문가(의사) 추천 연계</t>
         </is>
       </c>
       <c r="C29" s="49" t="inlineStr">
         <is>
-          <t>10월 예열 + 11월 D-day</t>
+          <t>7~10월 KOL 주기 배포</t>
         </is>
       </c>
       <c r="D29" s="25" t="inlineStr"/>
@@ -2093,15 +2049,19 @@
       <c r="G29" s="25" t="inlineStr"/>
       <c r="H29" s="25" t="inlineStr"/>
       <c r="I29" s="25" t="inlineStr"/>
-      <c r="J29" s="25" t="inlineStr"/>
-      <c r="K29" s="25" t="inlineStr"/>
-      <c r="L29" s="25" t="inlineStr"/>
+      <c r="J29" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="K29" s="50" t="n">
+        <v>25</v>
+      </c>
+      <c r="L29" s="50" t="n">
+        <v>25</v>
+      </c>
       <c r="M29" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="N29" s="50" t="n">
-        <v>60</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="N29" s="25" t="inlineStr"/>
       <c r="O29" s="25" t="inlineStr"/>
       <c r="P29" s="51" t="n">
         <v>80</v>
@@ -2111,12 +2071,12 @@
       <c r="A30" s="47" t="inlineStr"/>
       <c r="B30" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 쌍12 (12/12) 연말 마감 캠페인</t>
+          <t xml:space="preserve"> 광군절 11.11 집중 캠페인</t>
         </is>
       </c>
       <c r="C30" s="49" t="inlineStr">
         <is>
-          <t>연간 목표 달성 마감</t>
+          <t>10월 예열 + 11월 D-day</t>
         </is>
       </c>
       <c r="D30" s="25" t="inlineStr"/>
@@ -2128,25 +2088,27 @@
       <c r="J30" s="25" t="inlineStr"/>
       <c r="K30" s="25" t="inlineStr"/>
       <c r="L30" s="25" t="inlineStr"/>
-      <c r="M30" s="25" t="inlineStr"/>
-      <c r="N30" s="25" t="inlineStr"/>
-      <c r="O30" s="50" t="n">
-        <v>30</v>
-      </c>
+      <c r="M30" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="N30" s="50" t="n">
+        <v>60</v>
+      </c>
+      <c r="O30" s="25" t="inlineStr"/>
       <c r="P30" s="51" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="47" t="inlineStr"/>
       <c r="B31" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 화룬강중 (신규) 런칭 지원</t>
+          <t xml:space="preserve"> 쌍12 (12/12) 연말 마감 캠페인</t>
         </is>
       </c>
       <c r="C31" s="49" t="inlineStr">
         <is>
-          <t>800 파이프라인 / 런칭 예산 우선 배정 / 케이코스메몰 축소분 재배분</t>
+          <t>연간 목표 달성 마감</t>
         </is>
       </c>
       <c r="D31" s="25" t="inlineStr"/>
@@ -2154,121 +2116,117 @@
       <c r="F31" s="25" t="inlineStr"/>
       <c r="G31" s="25" t="inlineStr"/>
       <c r="H31" s="25" t="inlineStr"/>
-      <c r="I31" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="J31" s="50" t="n">
-        <v>5</v>
-      </c>
-      <c r="K31" s="50" t="n">
-        <v>5</v>
-      </c>
+      <c r="I31" s="25" t="inlineStr"/>
+      <c r="J31" s="25" t="inlineStr"/>
+      <c r="K31" s="25" t="inlineStr"/>
       <c r="L31" s="25" t="inlineStr"/>
       <c r="M31" s="25" t="inlineStr"/>
       <c r="N31" s="25" t="inlineStr"/>
-      <c r="O31" s="25" t="inlineStr"/>
+      <c r="O31" s="50" t="n">
+        <v>30</v>
+      </c>
       <c r="P31" s="51" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="47" t="inlineStr"/>
+      <c r="B32" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 화룬강중 (신규) 런칭 지원</t>
+        </is>
+      </c>
+      <c r="C32" s="49" t="inlineStr">
+        <is>
+          <t>800 파이프라인 / 런칭 예산 우선 배정 / 케이코스메몰 축소분 재배분</t>
+        </is>
+      </c>
+      <c r="D32" s="25" t="inlineStr"/>
+      <c r="E32" s="25" t="inlineStr"/>
+      <c r="F32" s="25" t="inlineStr"/>
+      <c r="G32" s="25" t="inlineStr"/>
+      <c r="H32" s="25" t="inlineStr"/>
+      <c r="I32" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="J32" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="L32" s="25" t="inlineStr"/>
+      <c r="M32" s="25" t="inlineStr"/>
+      <c r="N32" s="25" t="inlineStr"/>
+      <c r="O32" s="25" t="inlineStr"/>
+      <c r="P32" s="51" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="52" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="52" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr"/>
-      <c r="D32" s="18" t="inlineStr"/>
-      <c r="E32" s="18" t="inlineStr"/>
-      <c r="F32" s="18" t="inlineStr"/>
-      <c r="G32" s="18" t="inlineStr"/>
-      <c r="H32" s="18" t="inlineStr"/>
-      <c r="I32" s="18" t="n">
+      <c r="C33" s="17" t="inlineStr"/>
+      <c r="D33" s="18" t="inlineStr"/>
+      <c r="E33" s="18" t="inlineStr"/>
+      <c r="F33" s="18" t="inlineStr"/>
+      <c r="G33" s="18" t="inlineStr"/>
+      <c r="H33" s="18" t="inlineStr"/>
+      <c r="I33" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="J32" s="18" t="n">
+      <c r="J33" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="K32" s="18" t="n">
+      <c r="K33" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="L32" s="18" t="n">
+      <c r="L33" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="M32" s="18" t="n">
+      <c r="M33" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="N32" s="18" t="n">
+      <c r="N33" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="O32" s="18" t="n">
+      <c r="O33" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="P32" s="19" t="n">
+      <c r="P33" s="19" t="n">
         <v>270</v>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>대만</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>▶ 목표: 최종목표: 음료시장 성수기 집중 + Medfirst GP Top3 달성</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="53" t="inlineStr"/>
-      <c r="B34" s="54" t="inlineStr">
-        <is>
-          <t>️ 여름 음료 성수기 집중 광고 (7~9월)</t>
-        </is>
-      </c>
-      <c r="C34" s="55" t="inlineStr">
-        <is>
-          <t>여름 건강음료 수요 피크 시즌</t>
-        </is>
-      </c>
-      <c r="D34" s="25" t="inlineStr"/>
-      <c r="E34" s="25" t="inlineStr"/>
-      <c r="F34" s="25" t="inlineStr"/>
-      <c r="G34" s="25" t="inlineStr"/>
-      <c r="H34" s="25" t="inlineStr"/>
-      <c r="I34" s="25" t="inlineStr"/>
-      <c r="J34" s="56" t="n">
-        <v>20</v>
-      </c>
-      <c r="K34" s="56" t="n">
-        <v>25</v>
-      </c>
-      <c r="L34" s="56" t="n">
-        <v>15</v>
-      </c>
-      <c r="M34" s="25" t="inlineStr"/>
-      <c r="N34" s="25" t="inlineStr"/>
-      <c r="O34" s="25" t="inlineStr"/>
-      <c r="P34" s="57" t="n">
-        <v>60</v>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>▶ 목표: 최종목표: Medfirst 단일채널 집중 부스팅 | 성수기 7~9월 극대화</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="53" t="inlineStr"/>
       <c r="B35" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Medfirst 전문약국 O4O 마케팅 (LINE→약국)</t>
+          <t xml:space="preserve"> Medfirst LINE OA + 성수기 디지털 광고</t>
         </is>
       </c>
       <c r="C35" s="55" t="inlineStr">
         <is>
-          <t>닥터 추천 마크 부착 후 집행</t>
+          <t>여름 건강음료 피크 / LINE 푸시 + FB/IG 타겟광고</t>
         </is>
       </c>
       <c r="D35" s="25" t="inlineStr"/>
@@ -2277,110 +2235,114 @@
       <c r="G35" s="25" t="inlineStr"/>
       <c r="H35" s="25" t="inlineStr"/>
       <c r="I35" s="25" t="inlineStr"/>
-      <c r="J35" s="25" t="inlineStr"/>
-      <c r="K35" s="25" t="inlineStr"/>
-      <c r="L35" s="25" t="inlineStr"/>
-      <c r="M35" s="56" t="n">
-        <v>10</v>
-      </c>
+      <c r="J35" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="K35" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="L35" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="M35" s="25" t="inlineStr"/>
       <c r="N35" s="25" t="inlineStr"/>
       <c r="O35" s="25" t="inlineStr"/>
       <c r="P35" s="57" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="28" t="inlineStr">
+      <c r="A36" s="53" t="inlineStr"/>
+      <c r="B36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 약사 교육 키트 + POP물 + 성과 인센티브</t>
+        </is>
+      </c>
+      <c r="C36" s="55" t="inlineStr">
+        <is>
+          <t>약사 추천율 제고 / 처방 카드+선반 스티커 전점 설치</t>
+        </is>
+      </c>
+      <c r="D36" s="25" t="inlineStr"/>
+      <c r="E36" s="25" t="inlineStr"/>
+      <c r="F36" s="25" t="inlineStr"/>
+      <c r="G36" s="25" t="inlineStr"/>
+      <c r="H36" s="25" t="inlineStr"/>
+      <c r="I36" s="25" t="inlineStr"/>
+      <c r="J36" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="K36" s="25" t="inlineStr"/>
+      <c r="L36" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="M36" s="25" t="inlineStr"/>
+      <c r="N36" s="25" t="inlineStr"/>
+      <c r="O36" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="P36" s="57" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="28" t="inlineStr">
         <is>
           <t>대만</t>
         </is>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr"/>
-      <c r="D36" s="18" t="inlineStr"/>
-      <c r="E36" s="18" t="inlineStr"/>
-      <c r="F36" s="18" t="inlineStr"/>
-      <c r="G36" s="18" t="inlineStr"/>
-      <c r="H36" s="18" t="inlineStr"/>
-      <c r="I36" s="18" t="inlineStr"/>
-      <c r="J36" s="18" t="n">
+      <c r="C37" s="17" t="inlineStr"/>
+      <c r="D37" s="18" t="inlineStr"/>
+      <c r="E37" s="18" t="inlineStr"/>
+      <c r="F37" s="18" t="inlineStr"/>
+      <c r="G37" s="18" t="inlineStr"/>
+      <c r="H37" s="18" t="inlineStr"/>
+      <c r="I37" s="18" t="inlineStr"/>
+      <c r="J37" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="K37" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="L37" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K36" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="L36" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="M36" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="N36" s="18" t="inlineStr"/>
-      <c r="O36" s="18" t="inlineStr"/>
-      <c r="P36" s="19" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="58" t="inlineStr">
+      <c r="M37" s="18" t="inlineStr"/>
+      <c r="N37" s="18" t="inlineStr"/>
+      <c r="O37" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="P37" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="58" t="inlineStr">
         <is>
           <t>몽골</t>
         </is>
       </c>
-      <c r="B37" s="59" t="inlineStr">
+      <c r="B38" s="59" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 현지 자체 브랜딩 지원 + 스포츠 마케팅 강화 | 베트남 골든 없음 → 인서트 영상 지원 전환</t>
         </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="60" t="inlineStr"/>
-      <c r="B38" s="61" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
-        </is>
-      </c>
-      <c r="C38" s="62" t="inlineStr">
-        <is>
-          <t>현지 파트너 주도 / 웰라이프 지원</t>
-        </is>
-      </c>
-      <c r="D38" s="25" t="inlineStr"/>
-      <c r="E38" s="25" t="inlineStr"/>
-      <c r="F38" s="25" t="inlineStr"/>
-      <c r="G38" s="25" t="inlineStr"/>
-      <c r="H38" s="25" t="inlineStr"/>
-      <c r="I38" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="J38" s="25" t="inlineStr"/>
-      <c r="K38" s="25" t="inlineStr"/>
-      <c r="L38" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="M38" s="25" t="inlineStr"/>
-      <c r="N38" s="25" t="inlineStr"/>
-      <c r="O38" s="63" t="n">
-        <v>10</v>
-      </c>
-      <c r="P38" s="64" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="60" t="inlineStr"/>
       <c r="B39" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 인서트 영상 제작 + 현지 배포 지원</t>
+          <t xml:space="preserve"> 스포츠 이벤트 협찬 (마라톤 수분섭취 조끼 등)</t>
         </is>
       </c>
       <c r="C39" s="62" t="inlineStr">
         <is>
-          <t>베트남 골든 채널 종료 → 몽골 자체 SNS 인서트로 전환</t>
+          <t>현지 파트너 주도 / 웰라이프 지원</t>
         </is>
       </c>
       <c r="D39" s="25" t="inlineStr"/>
@@ -2388,353 +2350,387 @@
       <c r="F39" s="25" t="inlineStr"/>
       <c r="G39" s="25" t="inlineStr"/>
       <c r="H39" s="25" t="inlineStr"/>
-      <c r="I39" s="25" t="inlineStr"/>
-      <c r="J39" s="63" t="n">
-        <v>20</v>
-      </c>
-      <c r="K39" s="63" t="n">
-        <v>20</v>
-      </c>
+      <c r="I39" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" s="25" t="inlineStr"/>
+      <c r="K39" s="25" t="inlineStr"/>
       <c r="L39" s="63" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M39" s="25" t="inlineStr"/>
       <c r="N39" s="25" t="inlineStr"/>
-      <c r="O39" s="25" t="inlineStr"/>
+      <c r="O39" s="63" t="n">
+        <v>10</v>
+      </c>
       <c r="P39" s="64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="60" t="inlineStr"/>
+      <c r="B40" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 인서트 영상 제작 + 현지 배포 지원</t>
+        </is>
+      </c>
+      <c r="C40" s="62" t="inlineStr">
+        <is>
+          <t>베트남 골든 채널 종료 → 몽골 자체 SNS 인서트로 전환</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="inlineStr"/>
+      <c r="E40" s="25" t="inlineStr"/>
+      <c r="F40" s="25" t="inlineStr"/>
+      <c r="G40" s="25" t="inlineStr"/>
+      <c r="H40" s="25" t="inlineStr"/>
+      <c r="I40" s="25" t="inlineStr"/>
+      <c r="J40" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="K40" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="L40" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="M40" s="25" t="inlineStr"/>
+      <c r="N40" s="25" t="inlineStr"/>
+      <c r="O40" s="25" t="inlineStr"/>
+      <c r="P40" s="64" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="65" t="inlineStr">
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="65" t="inlineStr">
         <is>
           <t>몽골</t>
         </is>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr"/>
-      <c r="D40" s="18" t="inlineStr"/>
-      <c r="E40" s="18" t="inlineStr"/>
-      <c r="F40" s="18" t="inlineStr"/>
-      <c r="G40" s="18" t="inlineStr"/>
-      <c r="H40" s="18" t="inlineStr"/>
-      <c r="I40" s="18" t="n">
+      <c r="C41" s="17" t="inlineStr"/>
+      <c r="D41" s="18" t="inlineStr"/>
+      <c r="E41" s="18" t="inlineStr"/>
+      <c r="F41" s="18" t="inlineStr"/>
+      <c r="G41" s="18" t="inlineStr"/>
+      <c r="H41" s="18" t="inlineStr"/>
+      <c r="I41" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J40" s="18" t="n">
+      <c r="J41" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="K40" s="18" t="n">
+      <c r="K41" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="L40" s="18" t="n">
+      <c r="L41" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="M40" s="18" t="inlineStr"/>
-      <c r="N40" s="18" t="inlineStr"/>
-      <c r="O40" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="P40" s="19" t="n">
+      <c r="M41" s="18" t="inlineStr"/>
+      <c r="N41" s="18" t="inlineStr"/>
+      <c r="O41" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="P41" s="19" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="58" t="inlineStr">
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="58" t="inlineStr">
         <is>
           <t>싱가포르</t>
         </is>
       </c>
-      <c r="B41" s="59" t="inlineStr">
+      <c r="B42" s="59" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 가디언 입점 매출 확대 + EXACTITUDE 리오더 촉진</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="66" t="inlineStr"/>
-      <c r="B42" s="67" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="66" t="inlineStr"/>
+      <c r="B43" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve"> 가디언 협업 확대 + 입점 지원</t>
         </is>
       </c>
-      <c r="C42" s="68" t="inlineStr">
+      <c r="C43" s="68" t="inlineStr">
         <is>
           <t>가디언 83개점 확장 / EXACTITUDE 샘플링+판촉 집중</t>
         </is>
       </c>
-      <c r="D42" s="25" t="inlineStr"/>
-      <c r="E42" s="25" t="inlineStr"/>
-      <c r="F42" s="25" t="inlineStr"/>
-      <c r="G42" s="25" t="inlineStr"/>
-      <c r="H42" s="25" t="inlineStr"/>
-      <c r="I42" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="J42" s="25" t="inlineStr"/>
-      <c r="K42" s="25" t="inlineStr"/>
-      <c r="L42" s="25" t="inlineStr"/>
-      <c r="M42" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="N42" s="25" t="inlineStr"/>
-      <c r="O42" s="25" t="inlineStr"/>
-      <c r="P42" s="70" t="n">
+      <c r="D43" s="25" t="inlineStr"/>
+      <c r="E43" s="25" t="inlineStr"/>
+      <c r="F43" s="25" t="inlineStr"/>
+      <c r="G43" s="25" t="inlineStr"/>
+      <c r="H43" s="25" t="inlineStr"/>
+      <c r="I43" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="J43" s="25" t="inlineStr"/>
+      <c r="K43" s="25" t="inlineStr"/>
+      <c r="L43" s="25" t="inlineStr"/>
+      <c r="M43" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="N43" s="25" t="inlineStr"/>
+      <c r="O43" s="25" t="inlineStr"/>
+      <c r="P43" s="70" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="65" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="65" t="inlineStr">
         <is>
           <t>싱가포르</t>
         </is>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr"/>
-      <c r="D43" s="18" t="inlineStr"/>
-      <c r="E43" s="18" t="inlineStr"/>
-      <c r="F43" s="18" t="inlineStr"/>
-      <c r="G43" s="18" t="inlineStr"/>
-      <c r="H43" s="18" t="inlineStr"/>
-      <c r="I43" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="J43" s="18" t="inlineStr"/>
-      <c r="K43" s="18" t="inlineStr"/>
-      <c r="L43" s="18" t="inlineStr"/>
-      <c r="M43" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="N43" s="18" t="inlineStr"/>
-      <c r="O43" s="18" t="inlineStr"/>
-      <c r="P43" s="19" t="n">
+      <c r="C44" s="17" t="inlineStr"/>
+      <c r="D44" s="18" t="inlineStr"/>
+      <c r="E44" s="18" t="inlineStr"/>
+      <c r="F44" s="18" t="inlineStr"/>
+      <c r="G44" s="18" t="inlineStr"/>
+      <c r="H44" s="18" t="inlineStr"/>
+      <c r="I44" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="J44" s="18" t="inlineStr"/>
+      <c r="K44" s="18" t="inlineStr"/>
+      <c r="L44" s="18" t="inlineStr"/>
+      <c r="M44" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="N44" s="18" t="inlineStr"/>
+      <c r="O44" s="18" t="inlineStr"/>
+      <c r="P44" s="19" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="71" t="inlineStr">
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="71" t="inlineStr">
         <is>
           <t>중동</t>
         </is>
       </c>
-      <c r="B44" s="72" t="inlineStr">
+      <c r="B45" s="72" t="inlineStr">
         <is>
           <t>▶ 목표:  시장 분위기 악화 → 광고 최소화 / FOC 재협상 병행</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="73" t="inlineStr"/>
-      <c r="B45" s="74" t="inlineStr">
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="73" t="inlineStr"/>
+      <c r="B46" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve"> Dermazone 최소 프로모 지원</t>
         </is>
       </c>
-      <c r="C45" s="75" t="inlineStr">
+      <c r="C46" s="75" t="inlineStr">
         <is>
           <t>현상 유지 / 추가 투자 없음</t>
         </is>
       </c>
-      <c r="D45" s="25" t="inlineStr"/>
-      <c r="E45" s="25" t="inlineStr"/>
-      <c r="F45" s="25" t="inlineStr"/>
-      <c r="G45" s="25" t="inlineStr"/>
-      <c r="H45" s="25" t="inlineStr"/>
-      <c r="I45" s="76" t="n">
+      <c r="D46" s="25" t="inlineStr"/>
+      <c r="E46" s="25" t="inlineStr"/>
+      <c r="F46" s="25" t="inlineStr"/>
+      <c r="G46" s="25" t="inlineStr"/>
+      <c r="H46" s="25" t="inlineStr"/>
+      <c r="I46" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="J45" s="25" t="inlineStr"/>
-      <c r="K45" s="25" t="inlineStr"/>
-      <c r="L45" s="25" t="inlineStr"/>
-      <c r="M45" s="25" t="inlineStr"/>
-      <c r="N45" s="25" t="inlineStr"/>
-      <c r="O45" s="25" t="inlineStr"/>
-      <c r="P45" s="77" t="n">
+      <c r="J46" s="25" t="inlineStr"/>
+      <c r="K46" s="25" t="inlineStr"/>
+      <c r="L46" s="25" t="inlineStr"/>
+      <c r="M46" s="25" t="inlineStr"/>
+      <c r="N46" s="25" t="inlineStr"/>
+      <c r="O46" s="25" t="inlineStr"/>
+      <c r="P46" s="77" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="78" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="78" t="inlineStr">
         <is>
           <t>중동</t>
         </is>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr"/>
-      <c r="D46" s="18" t="inlineStr"/>
-      <c r="E46" s="18" t="inlineStr"/>
-      <c r="F46" s="18" t="inlineStr"/>
-      <c r="G46" s="18" t="inlineStr"/>
-      <c r="H46" s="18" t="inlineStr"/>
-      <c r="I46" s="18" t="n">
+      <c r="C47" s="17" t="inlineStr"/>
+      <c r="D47" s="18" t="inlineStr"/>
+      <c r="E47" s="18" t="inlineStr"/>
+      <c r="F47" s="18" t="inlineStr"/>
+      <c r="G47" s="18" t="inlineStr"/>
+      <c r="H47" s="18" t="inlineStr"/>
+      <c r="I47" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J46" s="18" t="inlineStr"/>
-      <c r="K46" s="18" t="inlineStr"/>
-      <c r="L46" s="18" t="inlineStr"/>
-      <c r="M46" s="18" t="inlineStr"/>
-      <c r="N46" s="18" t="inlineStr"/>
-      <c r="O46" s="18" t="inlineStr"/>
-      <c r="P46" s="19" t="n">
+      <c r="J47" s="18" t="inlineStr"/>
+      <c r="K47" s="18" t="inlineStr"/>
+      <c r="L47" s="18" t="inlineStr"/>
+      <c r="M47" s="18" t="inlineStr"/>
+      <c r="N47" s="18" t="inlineStr"/>
+      <c r="O47" s="18" t="inlineStr"/>
+      <c r="P47" s="19" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="79" t="inlineStr">
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="79" t="inlineStr">
         <is>
           <t>호주</t>
         </is>
       </c>
-      <c r="B47" s="80" t="inlineStr">
+      <c r="B48" s="80" t="inlineStr">
         <is>
           <t>▶ 목표: 최종목표: 대상 호주 채널 안정화 (천호케어 제외 / 비용대비 성장률 없음)</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="81" t="inlineStr"/>
-      <c r="B48" s="82" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="81" t="inlineStr"/>
+      <c r="B49" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve"> 대상 호주 공동 마케팅 지원</t>
         </is>
       </c>
-      <c r="C48" s="83" t="inlineStr">
+      <c r="C49" s="83" t="inlineStr">
         <is>
           <t>천호케어 제외 / 대상 호주 직접 채널만 지원</t>
         </is>
       </c>
-      <c r="D48" s="25" t="inlineStr"/>
-      <c r="E48" s="25" t="inlineStr"/>
-      <c r="F48" s="25" t="inlineStr"/>
-      <c r="G48" s="25" t="inlineStr"/>
-      <c r="H48" s="25" t="inlineStr"/>
-      <c r="I48" s="84" t="n">
+      <c r="D49" s="25" t="inlineStr"/>
+      <c r="E49" s="25" t="inlineStr"/>
+      <c r="F49" s="25" t="inlineStr"/>
+      <c r="G49" s="25" t="inlineStr"/>
+      <c r="H49" s="25" t="inlineStr"/>
+      <c r="I49" s="84" t="n">
         <v>5</v>
       </c>
-      <c r="J48" s="25" t="inlineStr"/>
-      <c r="K48" s="25" t="inlineStr"/>
-      <c r="L48" s="84" t="n">
+      <c r="J49" s="25" t="inlineStr"/>
+      <c r="K49" s="25" t="inlineStr"/>
+      <c r="L49" s="84" t="n">
         <v>5</v>
       </c>
-      <c r="M48" s="25" t="inlineStr"/>
-      <c r="N48" s="25" t="inlineStr"/>
-      <c r="O48" s="25" t="inlineStr"/>
-      <c r="P48" s="85" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="86" t="inlineStr">
+      <c r="M49" s="25" t="inlineStr"/>
+      <c r="N49" s="25" t="inlineStr"/>
+      <c r="O49" s="25" t="inlineStr"/>
+      <c r="P49" s="85" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="86" t="inlineStr">
         <is>
           <t>호주</t>
         </is>
       </c>
-      <c r="B49" s="16" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C49" s="17" t="inlineStr"/>
-      <c r="D49" s="18" t="inlineStr"/>
-      <c r="E49" s="18" t="inlineStr"/>
-      <c r="F49" s="18" t="inlineStr"/>
-      <c r="G49" s="18" t="inlineStr"/>
-      <c r="H49" s="18" t="inlineStr"/>
-      <c r="I49" s="18" t="n">
+      <c r="C50" s="17" t="inlineStr"/>
+      <c r="D50" s="18" t="inlineStr"/>
+      <c r="E50" s="18" t="inlineStr"/>
+      <c r="F50" s="18" t="inlineStr"/>
+      <c r="G50" s="18" t="inlineStr"/>
+      <c r="H50" s="18" t="inlineStr"/>
+      <c r="I50" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="J49" s="18" t="inlineStr"/>
-      <c r="K49" s="18" t="inlineStr"/>
-      <c r="L49" s="18" t="n">
+      <c r="J50" s="18" t="inlineStr"/>
+      <c r="K50" s="18" t="inlineStr"/>
+      <c r="L50" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M49" s="18" t="inlineStr"/>
-      <c r="N49" s="18" t="inlineStr"/>
-      <c r="O49" s="18" t="inlineStr"/>
-      <c r="P49" s="19" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="87" t="inlineStr">
+      <c r="M50" s="18" t="inlineStr"/>
+      <c r="N50" s="18" t="inlineStr"/>
+      <c r="O50" s="18" t="inlineStr"/>
+      <c r="P50" s="19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="87" t="inlineStr">
         <is>
           <t>총 합계 (백만원)</t>
         </is>
       </c>
-      <c r="D50" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="E50" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="F50" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="G50" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="H50" s="88" t="n">
-        <v>10</v>
-      </c>
-      <c r="I50" s="88" t="n">
-        <v>265</v>
-      </c>
-      <c r="J50" s="88" t="n">
-        <v>265</v>
-      </c>
-      <c r="K50" s="88" t="n">
-        <v>300</v>
-      </c>
-      <c r="L50" s="88" t="n">
-        <v>235</v>
-      </c>
-      <c r="M50" s="88" t="n">
-        <v>145</v>
-      </c>
-      <c r="N50" s="88" t="n">
-        <v>165</v>
-      </c>
-      <c r="O50" s="88" t="n">
-        <v>75</v>
-      </c>
-      <c r="P50" s="89" t="n">
+      <c r="D51" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="E51" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="F51" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="G51" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="H51" s="88" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" s="88" t="n">
+        <v>310</v>
+      </c>
+      <c r="J51" s="88" t="n">
+        <v>297</v>
+      </c>
+      <c r="K51" s="88" t="n">
+        <v>303</v>
+      </c>
+      <c r="L51" s="88" t="n">
+        <v>240</v>
+      </c>
+      <c r="M51" s="88" t="n">
+        <v>95</v>
+      </c>
+      <c r="N51" s="88" t="n">
+        <v>135</v>
+      </c>
+      <c r="O51" s="88" t="n">
+        <v>70</v>
+      </c>
+      <c r="P51" s="89" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 315  |  하반기(7~12월) 합계: 1,185  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ※ 총 집행 예산 1,500백만원  |  목표 15억원 대비 100.0%  |  상반기(1~6월) 합계: 360  |  하반기(7~12월) 합계: 1,140  |  주요 집중월: 6월(618) / 9월(중추절) / 11월(광군절·블프)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A51:P51"/>
     <mergeCell ref="B15:P15"/>
     <mergeCell ref="B7:P7"/>
-    <mergeCell ref="B33:P33"/>
-    <mergeCell ref="B44:P44"/>
-    <mergeCell ref="B47:P47"/>
+    <mergeCell ref="B38:P38"/>
+    <mergeCell ref="B48:P48"/>
+    <mergeCell ref="B34:P34"/>
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="B37:P37"/>
-    <mergeCell ref="B41:P41"/>
+    <mergeCell ref="B42:P42"/>
+    <mergeCell ref="B22:P22"/>
+    <mergeCell ref="B45:P45"/>
+    <mergeCell ref="B27:P27"/>
     <mergeCell ref="B4:P4"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="B26:P26"/>
-    <mergeCell ref="B21:P21"/>
+    <mergeCell ref="A52:P52"/>
+    <mergeCell ref="A51:C51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>